<commit_message>
Update Pertanggal 20 Mei 2026 15:16 WIB
</commit_message>
<xml_diff>
--- a/Documentation/Documents/SQL Generator/Data Initial/SysConfig.TblAppObject_MenuGroupMember.xlsx
+++ b/Documentation/Documents/SQL Generator/Data Initial/SysConfig.TblAppObject_MenuGroupMember.xlsx
@@ -1728,10 +1728,10 @@
 "'sysPartitionRemovableRecordKey_RefID', NULL::bigint,",
 "'sysBranch_RefID', varInstitutionBranchID::bigint,",
 "'sysBaseCurrency_RefID',varBaseCurrencyID::bigint,",
-"'name', ", IF(EXACT($G2, ""), "null", CONCATENATE("'", SUBSTITUTE($G2, "'", "\'"), "'")), "::varchar,",
-"'iconSource', ", IF(EXACT($B2, ""), "null", CONCATENATE("'", SUBSTITUTE($B2, "'", "\'"), "'")), "::varchar",
+"'menuGroup_RefID', ", IF(EXACT($G2, ""), "null", CONCATENATE("'", SUBSTITUTE($G2, "'", "\'"), "'")), "::bigint,",
+"'menu_RefID', ", IF(EXACT($B2, ""), "null", CONCATENATE("'", SUBSTITUTE($B2, "'", "\'"), "'")), "::bigint",
 ")))::varchar;")</f>
-        <v>varSQL := varSQL || (CASE WHEN (varSQL = '') THEN '' ELSE ', ' END) || (SELECT JSON_BUILD_OBJECT ('recordID', NULL::bigint,'entities', JSON_BUILD_OBJECT ('sysLoginSession_RefID', varSystemLoginSession::bigint,'sysDataAnnotation', NULL::varchar,'sysDataSetDateTimeTZ', NULL::timestamptz,'sysDataValidityStartDateTimeTZ', NULL::timestamptz,'sysDataValidityFinishDateTimeTZ', NULL::timestamptz,'sysPartitionRemovableRecordKey_RefID', NULL::bigint,'sysBranch_RefID', varInstitutionBranchID::bigint,'sysBaseCurrency_RefID',varBaseCurrencyID::bigint,'name', '254000000000001'::varchar,'iconSource', '97000000000001'::varchar)))::varchar;</v>
+        <v>varSQL := varSQL || (CASE WHEN (varSQL = '') THEN '' ELSE ', ' END) || (SELECT JSON_BUILD_OBJECT ('recordID', NULL::bigint,'entities', JSON_BUILD_OBJECT ('sysLoginSession_RefID', varSystemLoginSession::bigint,'sysDataAnnotation', NULL::varchar,'sysDataSetDateTimeTZ', NULL::timestamptz,'sysDataValidityStartDateTimeTZ', NULL::timestamptz,'sysDataValidityFinishDateTimeTZ', NULL::timestamptz,'sysPartitionRemovableRecordKey_RefID', NULL::bigint,'sysBranch_RefID', varInstitutionBranchID::bigint,'sysBaseCurrency_RefID',varBaseCurrencyID::bigint,'menuGroup_RefID', '254000000000001'::bigint,'menu_RefID', '97000000000001'::bigint)))::varchar;</v>
       </c>
     </row>
     <row r="3" spans="2:11" x14ac:dyDescent="0.2">
@@ -1773,10 +1773,10 @@
 "'sysPartitionRemovableRecordKey_RefID', NULL::bigint,",
 "'sysBranch_RefID', varInstitutionBranchID::bigint,",
 "'sysBaseCurrency_RefID',varBaseCurrencyID::bigint,",
-"'name', ", IF(EXACT($G3, ""), "null", CONCATENATE("'", SUBSTITUTE($G3, "'", "\'"), "'")), "::varchar,",
-"'iconSource', ", IF(EXACT($B3, ""), "null", CONCATENATE("'", SUBSTITUTE($B3, "'", "\'"), "'")), "::varchar",
+"'menuGroup_RefID', ", IF(EXACT($G3, ""), "null", CONCATENATE("'", SUBSTITUTE($G3, "'", "\'"), "'")), "::bigint,",
+"'menu_RefID', ", IF(EXACT($B3, ""), "null", CONCATENATE("'", SUBSTITUTE($B3, "'", "\'"), "'")), "::bigint",
 ")))::varchar;")</f>
-        <v>varSQL := varSQL || (CASE WHEN (varSQL = '') THEN '' ELSE ', ' END) || (SELECT JSON_BUILD_OBJECT ('recordID', NULL::bigint,'entities', JSON_BUILD_OBJECT ('sysLoginSession_RefID', varSystemLoginSession::bigint,'sysDataAnnotation', NULL::varchar,'sysDataSetDateTimeTZ', NULL::timestamptz,'sysDataValidityStartDateTimeTZ', NULL::timestamptz,'sysDataValidityFinishDateTimeTZ', NULL::timestamptz,'sysPartitionRemovableRecordKey_RefID', NULL::bigint,'sysBranch_RefID', varInstitutionBranchID::bigint,'sysBaseCurrency_RefID',varBaseCurrencyID::bigint,'name', '254000000000001'::varchar,'iconSource', '97000000000002'::varchar)))::varchar;</v>
+        <v>varSQL := varSQL || (CASE WHEN (varSQL = '') THEN '' ELSE ', ' END) || (SELECT JSON_BUILD_OBJECT ('recordID', NULL::bigint,'entities', JSON_BUILD_OBJECT ('sysLoginSession_RefID', varSystemLoginSession::bigint,'sysDataAnnotation', NULL::varchar,'sysDataSetDateTimeTZ', NULL::timestamptz,'sysDataValidityStartDateTimeTZ', NULL::timestamptz,'sysDataValidityFinishDateTimeTZ', NULL::timestamptz,'sysPartitionRemovableRecordKey_RefID', NULL::bigint,'sysBranch_RefID', varInstitutionBranchID::bigint,'sysBaseCurrency_RefID',varBaseCurrencyID::bigint,'menuGroup_RefID', '254000000000001'::bigint,'menu_RefID', '97000000000002'::bigint)))::varchar;</v>
       </c>
     </row>
     <row r="4" spans="2:11" x14ac:dyDescent="0.2">
@@ -1808,7 +1808,7 @@
       </c>
       <c r="K4" s="2" t="str">
         <f t="shared" si="1"/>
-        <v>varSQL := varSQL || (CASE WHEN (varSQL = '') THEN '' ELSE ', ' END) || (SELECT JSON_BUILD_OBJECT ('recordID', NULL::bigint,'entities', JSON_BUILD_OBJECT ('sysLoginSession_RefID', varSystemLoginSession::bigint,'sysDataAnnotation', NULL::varchar,'sysDataSetDateTimeTZ', NULL::timestamptz,'sysDataValidityStartDateTimeTZ', NULL::timestamptz,'sysDataValidityFinishDateTimeTZ', NULL::timestamptz,'sysPartitionRemovableRecordKey_RefID', NULL::bigint,'sysBranch_RefID', varInstitutionBranchID::bigint,'sysBaseCurrency_RefID',varBaseCurrencyID::bigint,'name', '254000000000001'::varchar,'iconSource', '97000000000003'::varchar)))::varchar;</v>
+        <v>varSQL := varSQL || (CASE WHEN (varSQL = '') THEN '' ELSE ', ' END) || (SELECT JSON_BUILD_OBJECT ('recordID', NULL::bigint,'entities', JSON_BUILD_OBJECT ('sysLoginSession_RefID', varSystemLoginSession::bigint,'sysDataAnnotation', NULL::varchar,'sysDataSetDateTimeTZ', NULL::timestamptz,'sysDataValidityStartDateTimeTZ', NULL::timestamptz,'sysDataValidityFinishDateTimeTZ', NULL::timestamptz,'sysPartitionRemovableRecordKey_RefID', NULL::bigint,'sysBranch_RefID', varInstitutionBranchID::bigint,'sysBaseCurrency_RefID',varBaseCurrencyID::bigint,'menuGroup_RefID', '254000000000001'::bigint,'menu_RefID', '97000000000003'::bigint)))::varchar;</v>
       </c>
     </row>
     <row r="5" spans="2:11" x14ac:dyDescent="0.2">
@@ -1840,7 +1840,7 @@
       </c>
       <c r="K5" s="2" t="str">
         <f t="shared" si="1"/>
-        <v>varSQL := varSQL || (CASE WHEN (varSQL = '') THEN '' ELSE ', ' END) || (SELECT JSON_BUILD_OBJECT ('recordID', NULL::bigint,'entities', JSON_BUILD_OBJECT ('sysLoginSession_RefID', varSystemLoginSession::bigint,'sysDataAnnotation', NULL::varchar,'sysDataSetDateTimeTZ', NULL::timestamptz,'sysDataValidityStartDateTimeTZ', NULL::timestamptz,'sysDataValidityFinishDateTimeTZ', NULL::timestamptz,'sysPartitionRemovableRecordKey_RefID', NULL::bigint,'sysBranch_RefID', varInstitutionBranchID::bigint,'sysBaseCurrency_RefID',varBaseCurrencyID::bigint,'name', '254000000000001'::varchar,'iconSource', '97000000000004'::varchar)))::varchar;</v>
+        <v>varSQL := varSQL || (CASE WHEN (varSQL = '') THEN '' ELSE ', ' END) || (SELECT JSON_BUILD_OBJECT ('recordID', NULL::bigint,'entities', JSON_BUILD_OBJECT ('sysLoginSession_RefID', varSystemLoginSession::bigint,'sysDataAnnotation', NULL::varchar,'sysDataSetDateTimeTZ', NULL::timestamptz,'sysDataValidityStartDateTimeTZ', NULL::timestamptz,'sysDataValidityFinishDateTimeTZ', NULL::timestamptz,'sysPartitionRemovableRecordKey_RefID', NULL::bigint,'sysBranch_RefID', varInstitutionBranchID::bigint,'sysBaseCurrency_RefID',varBaseCurrencyID::bigint,'menuGroup_RefID', '254000000000001'::bigint,'menu_RefID', '97000000000004'::bigint)))::varchar;</v>
       </c>
     </row>
     <row r="6" spans="2:11" x14ac:dyDescent="0.2">
@@ -1872,7 +1872,7 @@
       </c>
       <c r="K6" s="2" t="str">
         <f t="shared" si="1"/>
-        <v>varSQL := varSQL || (CASE WHEN (varSQL = '') THEN '' ELSE ', ' END) || (SELECT JSON_BUILD_OBJECT ('recordID', NULL::bigint,'entities', JSON_BUILD_OBJECT ('sysLoginSession_RefID', varSystemLoginSession::bigint,'sysDataAnnotation', NULL::varchar,'sysDataSetDateTimeTZ', NULL::timestamptz,'sysDataValidityStartDateTimeTZ', NULL::timestamptz,'sysDataValidityFinishDateTimeTZ', NULL::timestamptz,'sysPartitionRemovableRecordKey_RefID', NULL::bigint,'sysBranch_RefID', varInstitutionBranchID::bigint,'sysBaseCurrency_RefID',varBaseCurrencyID::bigint,'name', '254000000000001'::varchar,'iconSource', '97000000000005'::varchar)))::varchar;</v>
+        <v>varSQL := varSQL || (CASE WHEN (varSQL = '') THEN '' ELSE ', ' END) || (SELECT JSON_BUILD_OBJECT ('recordID', NULL::bigint,'entities', JSON_BUILD_OBJECT ('sysLoginSession_RefID', varSystemLoginSession::bigint,'sysDataAnnotation', NULL::varchar,'sysDataSetDateTimeTZ', NULL::timestamptz,'sysDataValidityStartDateTimeTZ', NULL::timestamptz,'sysDataValidityFinishDateTimeTZ', NULL::timestamptz,'sysPartitionRemovableRecordKey_RefID', NULL::bigint,'sysBranch_RefID', varInstitutionBranchID::bigint,'sysBaseCurrency_RefID',varBaseCurrencyID::bigint,'menuGroup_RefID', '254000000000001'::bigint,'menu_RefID', '97000000000005'::bigint)))::varchar;</v>
       </c>
     </row>
     <row r="7" spans="2:11" x14ac:dyDescent="0.2">
@@ -1904,7 +1904,7 @@
       </c>
       <c r="K7" s="2" t="str">
         <f t="shared" si="1"/>
-        <v>varSQL := varSQL || (CASE WHEN (varSQL = '') THEN '' ELSE ', ' END) || (SELECT JSON_BUILD_OBJECT ('recordID', NULL::bigint,'entities', JSON_BUILD_OBJECT ('sysLoginSession_RefID', varSystemLoginSession::bigint,'sysDataAnnotation', NULL::varchar,'sysDataSetDateTimeTZ', NULL::timestamptz,'sysDataValidityStartDateTimeTZ', NULL::timestamptz,'sysDataValidityFinishDateTimeTZ', NULL::timestamptz,'sysPartitionRemovableRecordKey_RefID', NULL::bigint,'sysBranch_RefID', varInstitutionBranchID::bigint,'sysBaseCurrency_RefID',varBaseCurrencyID::bigint,'name', '254000000000001'::varchar,'iconSource', '97000000000006'::varchar)))::varchar;</v>
+        <v>varSQL := varSQL || (CASE WHEN (varSQL = '') THEN '' ELSE ', ' END) || (SELECT JSON_BUILD_OBJECT ('recordID', NULL::bigint,'entities', JSON_BUILD_OBJECT ('sysLoginSession_RefID', varSystemLoginSession::bigint,'sysDataAnnotation', NULL::varchar,'sysDataSetDateTimeTZ', NULL::timestamptz,'sysDataValidityStartDateTimeTZ', NULL::timestamptz,'sysDataValidityFinishDateTimeTZ', NULL::timestamptz,'sysPartitionRemovableRecordKey_RefID', NULL::bigint,'sysBranch_RefID', varInstitutionBranchID::bigint,'sysBaseCurrency_RefID',varBaseCurrencyID::bigint,'menuGroup_RefID', '254000000000001'::bigint,'menu_RefID', '97000000000006'::bigint)))::varchar;</v>
       </c>
     </row>
     <row r="8" spans="2:11" x14ac:dyDescent="0.2">
@@ -1936,7 +1936,7 @@
       </c>
       <c r="K8" s="2" t="str">
         <f t="shared" si="1"/>
-        <v>varSQL := varSQL || (CASE WHEN (varSQL = '') THEN '' ELSE ', ' END) || (SELECT JSON_BUILD_OBJECT ('recordID', NULL::bigint,'entities', JSON_BUILD_OBJECT ('sysLoginSession_RefID', varSystemLoginSession::bigint,'sysDataAnnotation', NULL::varchar,'sysDataSetDateTimeTZ', NULL::timestamptz,'sysDataValidityStartDateTimeTZ', NULL::timestamptz,'sysDataValidityFinishDateTimeTZ', NULL::timestamptz,'sysPartitionRemovableRecordKey_RefID', NULL::bigint,'sysBranch_RefID', varInstitutionBranchID::bigint,'sysBaseCurrency_RefID',varBaseCurrencyID::bigint,'name', '254000000000001'::varchar,'iconSource', '97000000000007'::varchar)))::varchar;</v>
+        <v>varSQL := varSQL || (CASE WHEN (varSQL = '') THEN '' ELSE ', ' END) || (SELECT JSON_BUILD_OBJECT ('recordID', NULL::bigint,'entities', JSON_BUILD_OBJECT ('sysLoginSession_RefID', varSystemLoginSession::bigint,'sysDataAnnotation', NULL::varchar,'sysDataSetDateTimeTZ', NULL::timestamptz,'sysDataValidityStartDateTimeTZ', NULL::timestamptz,'sysDataValidityFinishDateTimeTZ', NULL::timestamptz,'sysPartitionRemovableRecordKey_RefID', NULL::bigint,'sysBranch_RefID', varInstitutionBranchID::bigint,'sysBaseCurrency_RefID',varBaseCurrencyID::bigint,'menuGroup_RefID', '254000000000001'::bigint,'menu_RefID', '97000000000007'::bigint)))::varchar;</v>
       </c>
     </row>
     <row r="9" spans="2:11" x14ac:dyDescent="0.2">
@@ -1968,7 +1968,7 @@
       </c>
       <c r="K9" s="2" t="str">
         <f t="shared" si="1"/>
-        <v>varSQL := varSQL || (CASE WHEN (varSQL = '') THEN '' ELSE ', ' END) || (SELECT JSON_BUILD_OBJECT ('recordID', NULL::bigint,'entities', JSON_BUILD_OBJECT ('sysLoginSession_RefID', varSystemLoginSession::bigint,'sysDataAnnotation', NULL::varchar,'sysDataSetDateTimeTZ', NULL::timestamptz,'sysDataValidityStartDateTimeTZ', NULL::timestamptz,'sysDataValidityFinishDateTimeTZ', NULL::timestamptz,'sysPartitionRemovableRecordKey_RefID', NULL::bigint,'sysBranch_RefID', varInstitutionBranchID::bigint,'sysBaseCurrency_RefID',varBaseCurrencyID::bigint,'name', '254000000000002'::varchar,'iconSource', '97000000000008'::varchar)))::varchar;</v>
+        <v>varSQL := varSQL || (CASE WHEN (varSQL = '') THEN '' ELSE ', ' END) || (SELECT JSON_BUILD_OBJECT ('recordID', NULL::bigint,'entities', JSON_BUILD_OBJECT ('sysLoginSession_RefID', varSystemLoginSession::bigint,'sysDataAnnotation', NULL::varchar,'sysDataSetDateTimeTZ', NULL::timestamptz,'sysDataValidityStartDateTimeTZ', NULL::timestamptz,'sysDataValidityFinishDateTimeTZ', NULL::timestamptz,'sysPartitionRemovableRecordKey_RefID', NULL::bigint,'sysBranch_RefID', varInstitutionBranchID::bigint,'sysBaseCurrency_RefID',varBaseCurrencyID::bigint,'menuGroup_RefID', '254000000000002'::bigint,'menu_RefID', '97000000000008'::bigint)))::varchar;</v>
       </c>
     </row>
     <row r="10" spans="2:11" x14ac:dyDescent="0.2">
@@ -2000,7 +2000,7 @@
       </c>
       <c r="K10" s="2" t="str">
         <f t="shared" si="1"/>
-        <v>varSQL := varSQL || (CASE WHEN (varSQL = '') THEN '' ELSE ', ' END) || (SELECT JSON_BUILD_OBJECT ('recordID', NULL::bigint,'entities', JSON_BUILD_OBJECT ('sysLoginSession_RefID', varSystemLoginSession::bigint,'sysDataAnnotation', NULL::varchar,'sysDataSetDateTimeTZ', NULL::timestamptz,'sysDataValidityStartDateTimeTZ', NULL::timestamptz,'sysDataValidityFinishDateTimeTZ', NULL::timestamptz,'sysPartitionRemovableRecordKey_RefID', NULL::bigint,'sysBranch_RefID', varInstitutionBranchID::bigint,'sysBaseCurrency_RefID',varBaseCurrencyID::bigint,'name', '254000000000002'::varchar,'iconSource', '97000000000009'::varchar)))::varchar;</v>
+        <v>varSQL := varSQL || (CASE WHEN (varSQL = '') THEN '' ELSE ', ' END) || (SELECT JSON_BUILD_OBJECT ('recordID', NULL::bigint,'entities', JSON_BUILD_OBJECT ('sysLoginSession_RefID', varSystemLoginSession::bigint,'sysDataAnnotation', NULL::varchar,'sysDataSetDateTimeTZ', NULL::timestamptz,'sysDataValidityStartDateTimeTZ', NULL::timestamptz,'sysDataValidityFinishDateTimeTZ', NULL::timestamptz,'sysPartitionRemovableRecordKey_RefID', NULL::bigint,'sysBranch_RefID', varInstitutionBranchID::bigint,'sysBaseCurrency_RefID',varBaseCurrencyID::bigint,'menuGroup_RefID', '254000000000002'::bigint,'menu_RefID', '97000000000009'::bigint)))::varchar;</v>
       </c>
     </row>
     <row r="11" spans="2:11" x14ac:dyDescent="0.2">
@@ -2032,7 +2032,7 @@
       </c>
       <c r="K11" s="2" t="str">
         <f t="shared" si="1"/>
-        <v>varSQL := varSQL || (CASE WHEN (varSQL = '') THEN '' ELSE ', ' END) || (SELECT JSON_BUILD_OBJECT ('recordID', NULL::bigint,'entities', JSON_BUILD_OBJECT ('sysLoginSession_RefID', varSystemLoginSession::bigint,'sysDataAnnotation', NULL::varchar,'sysDataSetDateTimeTZ', NULL::timestamptz,'sysDataValidityStartDateTimeTZ', NULL::timestamptz,'sysDataValidityFinishDateTimeTZ', NULL::timestamptz,'sysPartitionRemovableRecordKey_RefID', NULL::bigint,'sysBranch_RefID', varInstitutionBranchID::bigint,'sysBaseCurrency_RefID',varBaseCurrencyID::bigint,'name', '254000000000002'::varchar,'iconSource', '97000000000010'::varchar)))::varchar;</v>
+        <v>varSQL := varSQL || (CASE WHEN (varSQL = '') THEN '' ELSE ', ' END) || (SELECT JSON_BUILD_OBJECT ('recordID', NULL::bigint,'entities', JSON_BUILD_OBJECT ('sysLoginSession_RefID', varSystemLoginSession::bigint,'sysDataAnnotation', NULL::varchar,'sysDataSetDateTimeTZ', NULL::timestamptz,'sysDataValidityStartDateTimeTZ', NULL::timestamptz,'sysDataValidityFinishDateTimeTZ', NULL::timestamptz,'sysPartitionRemovableRecordKey_RefID', NULL::bigint,'sysBranch_RefID', varInstitutionBranchID::bigint,'sysBaseCurrency_RefID',varBaseCurrencyID::bigint,'menuGroup_RefID', '254000000000002'::bigint,'menu_RefID', '97000000000010'::bigint)))::varchar;</v>
       </c>
     </row>
     <row r="12" spans="2:11" x14ac:dyDescent="0.2">
@@ -2064,7 +2064,7 @@
       </c>
       <c r="K12" s="2" t="str">
         <f t="shared" si="1"/>
-        <v>varSQL := varSQL || (CASE WHEN (varSQL = '') THEN '' ELSE ', ' END) || (SELECT JSON_BUILD_OBJECT ('recordID', NULL::bigint,'entities', JSON_BUILD_OBJECT ('sysLoginSession_RefID', varSystemLoginSession::bigint,'sysDataAnnotation', NULL::varchar,'sysDataSetDateTimeTZ', NULL::timestamptz,'sysDataValidityStartDateTimeTZ', NULL::timestamptz,'sysDataValidityFinishDateTimeTZ', NULL::timestamptz,'sysPartitionRemovableRecordKey_RefID', NULL::bigint,'sysBranch_RefID', varInstitutionBranchID::bigint,'sysBaseCurrency_RefID',varBaseCurrencyID::bigint,'name', '254000000000002'::varchar,'iconSource', '97000000000011'::varchar)))::varchar;</v>
+        <v>varSQL := varSQL || (CASE WHEN (varSQL = '') THEN '' ELSE ', ' END) || (SELECT JSON_BUILD_OBJECT ('recordID', NULL::bigint,'entities', JSON_BUILD_OBJECT ('sysLoginSession_RefID', varSystemLoginSession::bigint,'sysDataAnnotation', NULL::varchar,'sysDataSetDateTimeTZ', NULL::timestamptz,'sysDataValidityStartDateTimeTZ', NULL::timestamptz,'sysDataValidityFinishDateTimeTZ', NULL::timestamptz,'sysPartitionRemovableRecordKey_RefID', NULL::bigint,'sysBranch_RefID', varInstitutionBranchID::bigint,'sysBaseCurrency_RefID',varBaseCurrencyID::bigint,'menuGroup_RefID', '254000000000002'::bigint,'menu_RefID', '97000000000011'::bigint)))::varchar;</v>
       </c>
     </row>
     <row r="13" spans="2:11" x14ac:dyDescent="0.2">
@@ -2096,7 +2096,7 @@
       </c>
       <c r="K13" s="2" t="str">
         <f t="shared" si="1"/>
-        <v>varSQL := varSQL || (CASE WHEN (varSQL = '') THEN '' ELSE ', ' END) || (SELECT JSON_BUILD_OBJECT ('recordID', NULL::bigint,'entities', JSON_BUILD_OBJECT ('sysLoginSession_RefID', varSystemLoginSession::bigint,'sysDataAnnotation', NULL::varchar,'sysDataSetDateTimeTZ', NULL::timestamptz,'sysDataValidityStartDateTimeTZ', NULL::timestamptz,'sysDataValidityFinishDateTimeTZ', NULL::timestamptz,'sysPartitionRemovableRecordKey_RefID', NULL::bigint,'sysBranch_RefID', varInstitutionBranchID::bigint,'sysBaseCurrency_RefID',varBaseCurrencyID::bigint,'name', '254000000000002'::varchar,'iconSource', '97000000000012'::varchar)))::varchar;</v>
+        <v>varSQL := varSQL || (CASE WHEN (varSQL = '') THEN '' ELSE ', ' END) || (SELECT JSON_BUILD_OBJECT ('recordID', NULL::bigint,'entities', JSON_BUILD_OBJECT ('sysLoginSession_RefID', varSystemLoginSession::bigint,'sysDataAnnotation', NULL::varchar,'sysDataSetDateTimeTZ', NULL::timestamptz,'sysDataValidityStartDateTimeTZ', NULL::timestamptz,'sysDataValidityFinishDateTimeTZ', NULL::timestamptz,'sysPartitionRemovableRecordKey_RefID', NULL::bigint,'sysBranch_RefID', varInstitutionBranchID::bigint,'sysBaseCurrency_RefID',varBaseCurrencyID::bigint,'menuGroup_RefID', '254000000000002'::bigint,'menu_RefID', '97000000000012'::bigint)))::varchar;</v>
       </c>
     </row>
     <row r="14" spans="2:11" x14ac:dyDescent="0.2">
@@ -2128,7 +2128,7 @@
       </c>
       <c r="K14" s="2" t="str">
         <f t="shared" si="1"/>
-        <v>varSQL := varSQL || (CASE WHEN (varSQL = '') THEN '' ELSE ', ' END) || (SELECT JSON_BUILD_OBJECT ('recordID', NULL::bigint,'entities', JSON_BUILD_OBJECT ('sysLoginSession_RefID', varSystemLoginSession::bigint,'sysDataAnnotation', NULL::varchar,'sysDataSetDateTimeTZ', NULL::timestamptz,'sysDataValidityStartDateTimeTZ', NULL::timestamptz,'sysDataValidityFinishDateTimeTZ', NULL::timestamptz,'sysPartitionRemovableRecordKey_RefID', NULL::bigint,'sysBranch_RefID', varInstitutionBranchID::bigint,'sysBaseCurrency_RefID',varBaseCurrencyID::bigint,'name', '254000000000002'::varchar,'iconSource', '97000000000013'::varchar)))::varchar;</v>
+        <v>varSQL := varSQL || (CASE WHEN (varSQL = '') THEN '' ELSE ', ' END) || (SELECT JSON_BUILD_OBJECT ('recordID', NULL::bigint,'entities', JSON_BUILD_OBJECT ('sysLoginSession_RefID', varSystemLoginSession::bigint,'sysDataAnnotation', NULL::varchar,'sysDataSetDateTimeTZ', NULL::timestamptz,'sysDataValidityStartDateTimeTZ', NULL::timestamptz,'sysDataValidityFinishDateTimeTZ', NULL::timestamptz,'sysPartitionRemovableRecordKey_RefID', NULL::bigint,'sysBranch_RefID', varInstitutionBranchID::bigint,'sysBaseCurrency_RefID',varBaseCurrencyID::bigint,'menuGroup_RefID', '254000000000002'::bigint,'menu_RefID', '97000000000013'::bigint)))::varchar;</v>
       </c>
     </row>
     <row r="15" spans="2:11" x14ac:dyDescent="0.2">
@@ -2160,7 +2160,7 @@
       </c>
       <c r="K15" s="2" t="str">
         <f t="shared" si="1"/>
-        <v>varSQL := varSQL || (CASE WHEN (varSQL = '') THEN '' ELSE ', ' END) || (SELECT JSON_BUILD_OBJECT ('recordID', NULL::bigint,'entities', JSON_BUILD_OBJECT ('sysLoginSession_RefID', varSystemLoginSession::bigint,'sysDataAnnotation', NULL::varchar,'sysDataSetDateTimeTZ', NULL::timestamptz,'sysDataValidityStartDateTimeTZ', NULL::timestamptz,'sysDataValidityFinishDateTimeTZ', NULL::timestamptz,'sysPartitionRemovableRecordKey_RefID', NULL::bigint,'sysBranch_RefID', varInstitutionBranchID::bigint,'sysBaseCurrency_RefID',varBaseCurrencyID::bigint,'name', '254000000000002'::varchar,'iconSource', '97000000000014'::varchar)))::varchar;</v>
+        <v>varSQL := varSQL || (CASE WHEN (varSQL = '') THEN '' ELSE ', ' END) || (SELECT JSON_BUILD_OBJECT ('recordID', NULL::bigint,'entities', JSON_BUILD_OBJECT ('sysLoginSession_RefID', varSystemLoginSession::bigint,'sysDataAnnotation', NULL::varchar,'sysDataSetDateTimeTZ', NULL::timestamptz,'sysDataValidityStartDateTimeTZ', NULL::timestamptz,'sysDataValidityFinishDateTimeTZ', NULL::timestamptz,'sysPartitionRemovableRecordKey_RefID', NULL::bigint,'sysBranch_RefID', varInstitutionBranchID::bigint,'sysBaseCurrency_RefID',varBaseCurrencyID::bigint,'menuGroup_RefID', '254000000000002'::bigint,'menu_RefID', '97000000000014'::bigint)))::varchar;</v>
       </c>
     </row>
     <row r="16" spans="2:11" x14ac:dyDescent="0.2">
@@ -2192,7 +2192,7 @@
       </c>
       <c r="K16" s="2" t="str">
         <f t="shared" si="1"/>
-        <v>varSQL := varSQL || (CASE WHEN (varSQL = '') THEN '' ELSE ', ' END) || (SELECT JSON_BUILD_OBJECT ('recordID', NULL::bigint,'entities', JSON_BUILD_OBJECT ('sysLoginSession_RefID', varSystemLoginSession::bigint,'sysDataAnnotation', NULL::varchar,'sysDataSetDateTimeTZ', NULL::timestamptz,'sysDataValidityStartDateTimeTZ', NULL::timestamptz,'sysDataValidityFinishDateTimeTZ', NULL::timestamptz,'sysPartitionRemovableRecordKey_RefID', NULL::bigint,'sysBranch_RefID', varInstitutionBranchID::bigint,'sysBaseCurrency_RefID',varBaseCurrencyID::bigint,'name', '254000000000002'::varchar,'iconSource', '97000000000015'::varchar)))::varchar;</v>
+        <v>varSQL := varSQL || (CASE WHEN (varSQL = '') THEN '' ELSE ', ' END) || (SELECT JSON_BUILD_OBJECT ('recordID', NULL::bigint,'entities', JSON_BUILD_OBJECT ('sysLoginSession_RefID', varSystemLoginSession::bigint,'sysDataAnnotation', NULL::varchar,'sysDataSetDateTimeTZ', NULL::timestamptz,'sysDataValidityStartDateTimeTZ', NULL::timestamptz,'sysDataValidityFinishDateTimeTZ', NULL::timestamptz,'sysPartitionRemovableRecordKey_RefID', NULL::bigint,'sysBranch_RefID', varInstitutionBranchID::bigint,'sysBaseCurrency_RefID',varBaseCurrencyID::bigint,'menuGroup_RefID', '254000000000002'::bigint,'menu_RefID', '97000000000015'::bigint)))::varchar;</v>
       </c>
     </row>
     <row r="17" spans="2:11" x14ac:dyDescent="0.2">
@@ -2224,7 +2224,7 @@
       </c>
       <c r="K17" s="2" t="str">
         <f t="shared" si="1"/>
-        <v>varSQL := varSQL || (CASE WHEN (varSQL = '') THEN '' ELSE ', ' END) || (SELECT JSON_BUILD_OBJECT ('recordID', NULL::bigint,'entities', JSON_BUILD_OBJECT ('sysLoginSession_RefID', varSystemLoginSession::bigint,'sysDataAnnotation', NULL::varchar,'sysDataSetDateTimeTZ', NULL::timestamptz,'sysDataValidityStartDateTimeTZ', NULL::timestamptz,'sysDataValidityFinishDateTimeTZ', NULL::timestamptz,'sysPartitionRemovableRecordKey_RefID', NULL::bigint,'sysBranch_RefID', varInstitutionBranchID::bigint,'sysBaseCurrency_RefID',varBaseCurrencyID::bigint,'name', '254000000000002'::varchar,'iconSource', '97000000000016'::varchar)))::varchar;</v>
+        <v>varSQL := varSQL || (CASE WHEN (varSQL = '') THEN '' ELSE ', ' END) || (SELECT JSON_BUILD_OBJECT ('recordID', NULL::bigint,'entities', JSON_BUILD_OBJECT ('sysLoginSession_RefID', varSystemLoginSession::bigint,'sysDataAnnotation', NULL::varchar,'sysDataSetDateTimeTZ', NULL::timestamptz,'sysDataValidityStartDateTimeTZ', NULL::timestamptz,'sysDataValidityFinishDateTimeTZ', NULL::timestamptz,'sysPartitionRemovableRecordKey_RefID', NULL::bigint,'sysBranch_RefID', varInstitutionBranchID::bigint,'sysBaseCurrency_RefID',varBaseCurrencyID::bigint,'menuGroup_RefID', '254000000000002'::bigint,'menu_RefID', '97000000000016'::bigint)))::varchar;</v>
       </c>
     </row>
     <row r="18" spans="2:11" x14ac:dyDescent="0.2">
@@ -2256,7 +2256,7 @@
       </c>
       <c r="K18" s="2" t="str">
         <f t="shared" si="1"/>
-        <v>varSQL := varSQL || (CASE WHEN (varSQL = '') THEN '' ELSE ', ' END) || (SELECT JSON_BUILD_OBJECT ('recordID', NULL::bigint,'entities', JSON_BUILD_OBJECT ('sysLoginSession_RefID', varSystemLoginSession::bigint,'sysDataAnnotation', NULL::varchar,'sysDataSetDateTimeTZ', NULL::timestamptz,'sysDataValidityStartDateTimeTZ', NULL::timestamptz,'sysDataValidityFinishDateTimeTZ', NULL::timestamptz,'sysPartitionRemovableRecordKey_RefID', NULL::bigint,'sysBranch_RefID', varInstitutionBranchID::bigint,'sysBaseCurrency_RefID',varBaseCurrencyID::bigint,'name', '254000000000002'::varchar,'iconSource', '97000000000017'::varchar)))::varchar;</v>
+        <v>varSQL := varSQL || (CASE WHEN (varSQL = '') THEN '' ELSE ', ' END) || (SELECT JSON_BUILD_OBJECT ('recordID', NULL::bigint,'entities', JSON_BUILD_OBJECT ('sysLoginSession_RefID', varSystemLoginSession::bigint,'sysDataAnnotation', NULL::varchar,'sysDataSetDateTimeTZ', NULL::timestamptz,'sysDataValidityStartDateTimeTZ', NULL::timestamptz,'sysDataValidityFinishDateTimeTZ', NULL::timestamptz,'sysPartitionRemovableRecordKey_RefID', NULL::bigint,'sysBranch_RefID', varInstitutionBranchID::bigint,'sysBaseCurrency_RefID',varBaseCurrencyID::bigint,'menuGroup_RefID', '254000000000002'::bigint,'menu_RefID', '97000000000017'::bigint)))::varchar;</v>
       </c>
     </row>
     <row r="19" spans="2:11" x14ac:dyDescent="0.2">
@@ -2288,7 +2288,7 @@
       </c>
       <c r="K19" s="2" t="str">
         <f t="shared" si="1"/>
-        <v>varSQL := varSQL || (CASE WHEN (varSQL = '') THEN '' ELSE ', ' END) || (SELECT JSON_BUILD_OBJECT ('recordID', NULL::bigint,'entities', JSON_BUILD_OBJECT ('sysLoginSession_RefID', varSystemLoginSession::bigint,'sysDataAnnotation', NULL::varchar,'sysDataSetDateTimeTZ', NULL::timestamptz,'sysDataValidityStartDateTimeTZ', NULL::timestamptz,'sysDataValidityFinishDateTimeTZ', NULL::timestamptz,'sysPartitionRemovableRecordKey_RefID', NULL::bigint,'sysBranch_RefID', varInstitutionBranchID::bigint,'sysBaseCurrency_RefID',varBaseCurrencyID::bigint,'name', '254000000000002'::varchar,'iconSource', '97000000000018'::varchar)))::varchar;</v>
+        <v>varSQL := varSQL || (CASE WHEN (varSQL = '') THEN '' ELSE ', ' END) || (SELECT JSON_BUILD_OBJECT ('recordID', NULL::bigint,'entities', JSON_BUILD_OBJECT ('sysLoginSession_RefID', varSystemLoginSession::bigint,'sysDataAnnotation', NULL::varchar,'sysDataSetDateTimeTZ', NULL::timestamptz,'sysDataValidityStartDateTimeTZ', NULL::timestamptz,'sysDataValidityFinishDateTimeTZ', NULL::timestamptz,'sysPartitionRemovableRecordKey_RefID', NULL::bigint,'sysBranch_RefID', varInstitutionBranchID::bigint,'sysBaseCurrency_RefID',varBaseCurrencyID::bigint,'menuGroup_RefID', '254000000000002'::bigint,'menu_RefID', '97000000000018'::bigint)))::varchar;</v>
       </c>
     </row>
     <row r="20" spans="2:11" x14ac:dyDescent="0.2">
@@ -2320,7 +2320,7 @@
       </c>
       <c r="K20" s="2" t="str">
         <f t="shared" si="1"/>
-        <v>varSQL := varSQL || (CASE WHEN (varSQL = '') THEN '' ELSE ', ' END) || (SELECT JSON_BUILD_OBJECT ('recordID', NULL::bigint,'entities', JSON_BUILD_OBJECT ('sysLoginSession_RefID', varSystemLoginSession::bigint,'sysDataAnnotation', NULL::varchar,'sysDataSetDateTimeTZ', NULL::timestamptz,'sysDataValidityStartDateTimeTZ', NULL::timestamptz,'sysDataValidityFinishDateTimeTZ', NULL::timestamptz,'sysPartitionRemovableRecordKey_RefID', NULL::bigint,'sysBranch_RefID', varInstitutionBranchID::bigint,'sysBaseCurrency_RefID',varBaseCurrencyID::bigint,'name', '254000000000004'::varchar,'iconSource', '97000000000019'::varchar)))::varchar;</v>
+        <v>varSQL := varSQL || (CASE WHEN (varSQL = '') THEN '' ELSE ', ' END) || (SELECT JSON_BUILD_OBJECT ('recordID', NULL::bigint,'entities', JSON_BUILD_OBJECT ('sysLoginSession_RefID', varSystemLoginSession::bigint,'sysDataAnnotation', NULL::varchar,'sysDataSetDateTimeTZ', NULL::timestamptz,'sysDataValidityStartDateTimeTZ', NULL::timestamptz,'sysDataValidityFinishDateTimeTZ', NULL::timestamptz,'sysPartitionRemovableRecordKey_RefID', NULL::bigint,'sysBranch_RefID', varInstitutionBranchID::bigint,'sysBaseCurrency_RefID',varBaseCurrencyID::bigint,'menuGroup_RefID', '254000000000004'::bigint,'menu_RefID', '97000000000019'::bigint)))::varchar;</v>
       </c>
     </row>
     <row r="21" spans="2:11" x14ac:dyDescent="0.2">
@@ -2352,7 +2352,7 @@
       </c>
       <c r="K21" s="2" t="str">
         <f t="shared" si="1"/>
-        <v>varSQL := varSQL || (CASE WHEN (varSQL = '') THEN '' ELSE ', ' END) || (SELECT JSON_BUILD_OBJECT ('recordID', NULL::bigint,'entities', JSON_BUILD_OBJECT ('sysLoginSession_RefID', varSystemLoginSession::bigint,'sysDataAnnotation', NULL::varchar,'sysDataSetDateTimeTZ', NULL::timestamptz,'sysDataValidityStartDateTimeTZ', NULL::timestamptz,'sysDataValidityFinishDateTimeTZ', NULL::timestamptz,'sysPartitionRemovableRecordKey_RefID', NULL::bigint,'sysBranch_RefID', varInstitutionBranchID::bigint,'sysBaseCurrency_RefID',varBaseCurrencyID::bigint,'name', '254000000000004'::varchar,'iconSource', '97000000000020'::varchar)))::varchar;</v>
+        <v>varSQL := varSQL || (CASE WHEN (varSQL = '') THEN '' ELSE ', ' END) || (SELECT JSON_BUILD_OBJECT ('recordID', NULL::bigint,'entities', JSON_BUILD_OBJECT ('sysLoginSession_RefID', varSystemLoginSession::bigint,'sysDataAnnotation', NULL::varchar,'sysDataSetDateTimeTZ', NULL::timestamptz,'sysDataValidityStartDateTimeTZ', NULL::timestamptz,'sysDataValidityFinishDateTimeTZ', NULL::timestamptz,'sysPartitionRemovableRecordKey_RefID', NULL::bigint,'sysBranch_RefID', varInstitutionBranchID::bigint,'sysBaseCurrency_RefID',varBaseCurrencyID::bigint,'menuGroup_RefID', '254000000000004'::bigint,'menu_RefID', '97000000000020'::bigint)))::varchar;</v>
       </c>
     </row>
     <row r="22" spans="2:11" x14ac:dyDescent="0.2">
@@ -2384,7 +2384,7 @@
       </c>
       <c r="K22" s="2" t="str">
         <f t="shared" si="1"/>
-        <v>varSQL := varSQL || (CASE WHEN (varSQL = '') THEN '' ELSE ', ' END) || (SELECT JSON_BUILD_OBJECT ('recordID', NULL::bigint,'entities', JSON_BUILD_OBJECT ('sysLoginSession_RefID', varSystemLoginSession::bigint,'sysDataAnnotation', NULL::varchar,'sysDataSetDateTimeTZ', NULL::timestamptz,'sysDataValidityStartDateTimeTZ', NULL::timestamptz,'sysDataValidityFinishDateTimeTZ', NULL::timestamptz,'sysPartitionRemovableRecordKey_RefID', NULL::bigint,'sysBranch_RefID', varInstitutionBranchID::bigint,'sysBaseCurrency_RefID',varBaseCurrencyID::bigint,'name', '254000000000004'::varchar,'iconSource', '97000000000021'::varchar)))::varchar;</v>
+        <v>varSQL := varSQL || (CASE WHEN (varSQL = '') THEN '' ELSE ', ' END) || (SELECT JSON_BUILD_OBJECT ('recordID', NULL::bigint,'entities', JSON_BUILD_OBJECT ('sysLoginSession_RefID', varSystemLoginSession::bigint,'sysDataAnnotation', NULL::varchar,'sysDataSetDateTimeTZ', NULL::timestamptz,'sysDataValidityStartDateTimeTZ', NULL::timestamptz,'sysDataValidityFinishDateTimeTZ', NULL::timestamptz,'sysPartitionRemovableRecordKey_RefID', NULL::bigint,'sysBranch_RefID', varInstitutionBranchID::bigint,'sysBaseCurrency_RefID',varBaseCurrencyID::bigint,'menuGroup_RefID', '254000000000004'::bigint,'menu_RefID', '97000000000021'::bigint)))::varchar;</v>
       </c>
     </row>
     <row r="23" spans="2:11" x14ac:dyDescent="0.2">
@@ -2416,7 +2416,7 @@
       </c>
       <c r="K23" s="2" t="str">
         <f t="shared" si="1"/>
-        <v>varSQL := varSQL || (CASE WHEN (varSQL = '') THEN '' ELSE ', ' END) || (SELECT JSON_BUILD_OBJECT ('recordID', NULL::bigint,'entities', JSON_BUILD_OBJECT ('sysLoginSession_RefID', varSystemLoginSession::bigint,'sysDataAnnotation', NULL::varchar,'sysDataSetDateTimeTZ', NULL::timestamptz,'sysDataValidityStartDateTimeTZ', NULL::timestamptz,'sysDataValidityFinishDateTimeTZ', NULL::timestamptz,'sysPartitionRemovableRecordKey_RefID', NULL::bigint,'sysBranch_RefID', varInstitutionBranchID::bigint,'sysBaseCurrency_RefID',varBaseCurrencyID::bigint,'name', '254000000000004'::varchar,'iconSource', '97000000000022'::varchar)))::varchar;</v>
+        <v>varSQL := varSQL || (CASE WHEN (varSQL = '') THEN '' ELSE ', ' END) || (SELECT JSON_BUILD_OBJECT ('recordID', NULL::bigint,'entities', JSON_BUILD_OBJECT ('sysLoginSession_RefID', varSystemLoginSession::bigint,'sysDataAnnotation', NULL::varchar,'sysDataSetDateTimeTZ', NULL::timestamptz,'sysDataValidityStartDateTimeTZ', NULL::timestamptz,'sysDataValidityFinishDateTimeTZ', NULL::timestamptz,'sysPartitionRemovableRecordKey_RefID', NULL::bigint,'sysBranch_RefID', varInstitutionBranchID::bigint,'sysBaseCurrency_RefID',varBaseCurrencyID::bigint,'menuGroup_RefID', '254000000000004'::bigint,'menu_RefID', '97000000000022'::bigint)))::varchar;</v>
       </c>
     </row>
     <row r="24" spans="2:11" x14ac:dyDescent="0.2">
@@ -2448,7 +2448,7 @@
       </c>
       <c r="K24" s="2" t="str">
         <f t="shared" si="1"/>
-        <v>varSQL := varSQL || (CASE WHEN (varSQL = '') THEN '' ELSE ', ' END) || (SELECT JSON_BUILD_OBJECT ('recordID', NULL::bigint,'entities', JSON_BUILD_OBJECT ('sysLoginSession_RefID', varSystemLoginSession::bigint,'sysDataAnnotation', NULL::varchar,'sysDataSetDateTimeTZ', NULL::timestamptz,'sysDataValidityStartDateTimeTZ', NULL::timestamptz,'sysDataValidityFinishDateTimeTZ', NULL::timestamptz,'sysPartitionRemovableRecordKey_RefID', NULL::bigint,'sysBranch_RefID', varInstitutionBranchID::bigint,'sysBaseCurrency_RefID',varBaseCurrencyID::bigint,'name', '254000000000004'::varchar,'iconSource', '97000000000023'::varchar)))::varchar;</v>
+        <v>varSQL := varSQL || (CASE WHEN (varSQL = '') THEN '' ELSE ', ' END) || (SELECT JSON_BUILD_OBJECT ('recordID', NULL::bigint,'entities', JSON_BUILD_OBJECT ('sysLoginSession_RefID', varSystemLoginSession::bigint,'sysDataAnnotation', NULL::varchar,'sysDataSetDateTimeTZ', NULL::timestamptz,'sysDataValidityStartDateTimeTZ', NULL::timestamptz,'sysDataValidityFinishDateTimeTZ', NULL::timestamptz,'sysPartitionRemovableRecordKey_RefID', NULL::bigint,'sysBranch_RefID', varInstitutionBranchID::bigint,'sysBaseCurrency_RefID',varBaseCurrencyID::bigint,'menuGroup_RefID', '254000000000004'::bigint,'menu_RefID', '97000000000023'::bigint)))::varchar;</v>
       </c>
     </row>
     <row r="25" spans="2:11" x14ac:dyDescent="0.2">
@@ -2480,7 +2480,7 @@
       </c>
       <c r="K25" s="2" t="str">
         <f t="shared" si="1"/>
-        <v>varSQL := varSQL || (CASE WHEN (varSQL = '') THEN '' ELSE ', ' END) || (SELECT JSON_BUILD_OBJECT ('recordID', NULL::bigint,'entities', JSON_BUILD_OBJECT ('sysLoginSession_RefID', varSystemLoginSession::bigint,'sysDataAnnotation', NULL::varchar,'sysDataSetDateTimeTZ', NULL::timestamptz,'sysDataValidityStartDateTimeTZ', NULL::timestamptz,'sysDataValidityFinishDateTimeTZ', NULL::timestamptz,'sysPartitionRemovableRecordKey_RefID', NULL::bigint,'sysBranch_RefID', varInstitutionBranchID::bigint,'sysBaseCurrency_RefID',varBaseCurrencyID::bigint,'name', '254000000000004'::varchar,'iconSource', '97000000000024'::varchar)))::varchar;</v>
+        <v>varSQL := varSQL || (CASE WHEN (varSQL = '') THEN '' ELSE ', ' END) || (SELECT JSON_BUILD_OBJECT ('recordID', NULL::bigint,'entities', JSON_BUILD_OBJECT ('sysLoginSession_RefID', varSystemLoginSession::bigint,'sysDataAnnotation', NULL::varchar,'sysDataSetDateTimeTZ', NULL::timestamptz,'sysDataValidityStartDateTimeTZ', NULL::timestamptz,'sysDataValidityFinishDateTimeTZ', NULL::timestamptz,'sysPartitionRemovableRecordKey_RefID', NULL::bigint,'sysBranch_RefID', varInstitutionBranchID::bigint,'sysBaseCurrency_RefID',varBaseCurrencyID::bigint,'menuGroup_RefID', '254000000000004'::bigint,'menu_RefID', '97000000000024'::bigint)))::varchar;</v>
       </c>
     </row>
     <row r="26" spans="2:11" x14ac:dyDescent="0.2">
@@ -2512,7 +2512,7 @@
       </c>
       <c r="K26" s="2" t="str">
         <f t="shared" si="1"/>
-        <v>varSQL := varSQL || (CASE WHEN (varSQL = '') THEN '' ELSE ', ' END) || (SELECT JSON_BUILD_OBJECT ('recordID', NULL::bigint,'entities', JSON_BUILD_OBJECT ('sysLoginSession_RefID', varSystemLoginSession::bigint,'sysDataAnnotation', NULL::varchar,'sysDataSetDateTimeTZ', NULL::timestamptz,'sysDataValidityStartDateTimeTZ', NULL::timestamptz,'sysDataValidityFinishDateTimeTZ', NULL::timestamptz,'sysPartitionRemovableRecordKey_RefID', NULL::bigint,'sysBranch_RefID', varInstitutionBranchID::bigint,'sysBaseCurrency_RefID',varBaseCurrencyID::bigint,'name', '254000000000007'::varchar,'iconSource', '97000000000025'::varchar)))::varchar;</v>
+        <v>varSQL := varSQL || (CASE WHEN (varSQL = '') THEN '' ELSE ', ' END) || (SELECT JSON_BUILD_OBJECT ('recordID', NULL::bigint,'entities', JSON_BUILD_OBJECT ('sysLoginSession_RefID', varSystemLoginSession::bigint,'sysDataAnnotation', NULL::varchar,'sysDataSetDateTimeTZ', NULL::timestamptz,'sysDataValidityStartDateTimeTZ', NULL::timestamptz,'sysDataValidityFinishDateTimeTZ', NULL::timestamptz,'sysPartitionRemovableRecordKey_RefID', NULL::bigint,'sysBranch_RefID', varInstitutionBranchID::bigint,'sysBaseCurrency_RefID',varBaseCurrencyID::bigint,'menuGroup_RefID', '254000000000007'::bigint,'menu_RefID', '97000000000025'::bigint)))::varchar;</v>
       </c>
     </row>
     <row r="27" spans="2:11" x14ac:dyDescent="0.2">
@@ -2544,7 +2544,7 @@
       </c>
       <c r="K27" s="2" t="str">
         <f t="shared" si="1"/>
-        <v>varSQL := varSQL || (CASE WHEN (varSQL = '') THEN '' ELSE ', ' END) || (SELECT JSON_BUILD_OBJECT ('recordID', NULL::bigint,'entities', JSON_BUILD_OBJECT ('sysLoginSession_RefID', varSystemLoginSession::bigint,'sysDataAnnotation', NULL::varchar,'sysDataSetDateTimeTZ', NULL::timestamptz,'sysDataValidityStartDateTimeTZ', NULL::timestamptz,'sysDataValidityFinishDateTimeTZ', NULL::timestamptz,'sysPartitionRemovableRecordKey_RefID', NULL::bigint,'sysBranch_RefID', varInstitutionBranchID::bigint,'sysBaseCurrency_RefID',varBaseCurrencyID::bigint,'name', '254000000000007'::varchar,'iconSource', '97000000000026'::varchar)))::varchar;</v>
+        <v>varSQL := varSQL || (CASE WHEN (varSQL = '') THEN '' ELSE ', ' END) || (SELECT JSON_BUILD_OBJECT ('recordID', NULL::bigint,'entities', JSON_BUILD_OBJECT ('sysLoginSession_RefID', varSystemLoginSession::bigint,'sysDataAnnotation', NULL::varchar,'sysDataSetDateTimeTZ', NULL::timestamptz,'sysDataValidityStartDateTimeTZ', NULL::timestamptz,'sysDataValidityFinishDateTimeTZ', NULL::timestamptz,'sysPartitionRemovableRecordKey_RefID', NULL::bigint,'sysBranch_RefID', varInstitutionBranchID::bigint,'sysBaseCurrency_RefID',varBaseCurrencyID::bigint,'menuGroup_RefID', '254000000000007'::bigint,'menu_RefID', '97000000000026'::bigint)))::varchar;</v>
       </c>
     </row>
     <row r="28" spans="2:11" x14ac:dyDescent="0.2">
@@ -2576,7 +2576,7 @@
       </c>
       <c r="K28" s="2" t="str">
         <f t="shared" si="1"/>
-        <v>varSQL := varSQL || (CASE WHEN (varSQL = '') THEN '' ELSE ', ' END) || (SELECT JSON_BUILD_OBJECT ('recordID', NULL::bigint,'entities', JSON_BUILD_OBJECT ('sysLoginSession_RefID', varSystemLoginSession::bigint,'sysDataAnnotation', NULL::varchar,'sysDataSetDateTimeTZ', NULL::timestamptz,'sysDataValidityStartDateTimeTZ', NULL::timestamptz,'sysDataValidityFinishDateTimeTZ', NULL::timestamptz,'sysPartitionRemovableRecordKey_RefID', NULL::bigint,'sysBranch_RefID', varInstitutionBranchID::bigint,'sysBaseCurrency_RefID',varBaseCurrencyID::bigint,'name', '254000000000007'::varchar,'iconSource', '97000000000027'::varchar)))::varchar;</v>
+        <v>varSQL := varSQL || (CASE WHEN (varSQL = '') THEN '' ELSE ', ' END) || (SELECT JSON_BUILD_OBJECT ('recordID', NULL::bigint,'entities', JSON_BUILD_OBJECT ('sysLoginSession_RefID', varSystemLoginSession::bigint,'sysDataAnnotation', NULL::varchar,'sysDataSetDateTimeTZ', NULL::timestamptz,'sysDataValidityStartDateTimeTZ', NULL::timestamptz,'sysDataValidityFinishDateTimeTZ', NULL::timestamptz,'sysPartitionRemovableRecordKey_RefID', NULL::bigint,'sysBranch_RefID', varInstitutionBranchID::bigint,'sysBaseCurrency_RefID',varBaseCurrencyID::bigint,'menuGroup_RefID', '254000000000007'::bigint,'menu_RefID', '97000000000027'::bigint)))::varchar;</v>
       </c>
     </row>
     <row r="29" spans="2:11" x14ac:dyDescent="0.2">
@@ -2608,7 +2608,7 @@
       </c>
       <c r="K29" s="2" t="str">
         <f t="shared" si="1"/>
-        <v>varSQL := varSQL || (CASE WHEN (varSQL = '') THEN '' ELSE ', ' END) || (SELECT JSON_BUILD_OBJECT ('recordID', NULL::bigint,'entities', JSON_BUILD_OBJECT ('sysLoginSession_RefID', varSystemLoginSession::bigint,'sysDataAnnotation', NULL::varchar,'sysDataSetDateTimeTZ', NULL::timestamptz,'sysDataValidityStartDateTimeTZ', NULL::timestamptz,'sysDataValidityFinishDateTimeTZ', NULL::timestamptz,'sysPartitionRemovableRecordKey_RefID', NULL::bigint,'sysBranch_RefID', varInstitutionBranchID::bigint,'sysBaseCurrency_RefID',varBaseCurrencyID::bigint,'name', '254000000000007'::varchar,'iconSource', '97000000000028'::varchar)))::varchar;</v>
+        <v>varSQL := varSQL || (CASE WHEN (varSQL = '') THEN '' ELSE ', ' END) || (SELECT JSON_BUILD_OBJECT ('recordID', NULL::bigint,'entities', JSON_BUILD_OBJECT ('sysLoginSession_RefID', varSystemLoginSession::bigint,'sysDataAnnotation', NULL::varchar,'sysDataSetDateTimeTZ', NULL::timestamptz,'sysDataValidityStartDateTimeTZ', NULL::timestamptz,'sysDataValidityFinishDateTimeTZ', NULL::timestamptz,'sysPartitionRemovableRecordKey_RefID', NULL::bigint,'sysBranch_RefID', varInstitutionBranchID::bigint,'sysBaseCurrency_RefID',varBaseCurrencyID::bigint,'menuGroup_RefID', '254000000000007'::bigint,'menu_RefID', '97000000000028'::bigint)))::varchar;</v>
       </c>
     </row>
     <row r="30" spans="2:11" x14ac:dyDescent="0.2">
@@ -2640,7 +2640,7 @@
       </c>
       <c r="K30" s="2" t="str">
         <f t="shared" si="1"/>
-        <v>varSQL := varSQL || (CASE WHEN (varSQL = '') THEN '' ELSE ', ' END) || (SELECT JSON_BUILD_OBJECT ('recordID', NULL::bigint,'entities', JSON_BUILD_OBJECT ('sysLoginSession_RefID', varSystemLoginSession::bigint,'sysDataAnnotation', NULL::varchar,'sysDataSetDateTimeTZ', NULL::timestamptz,'sysDataValidityStartDateTimeTZ', NULL::timestamptz,'sysDataValidityFinishDateTimeTZ', NULL::timestamptz,'sysPartitionRemovableRecordKey_RefID', NULL::bigint,'sysBranch_RefID', varInstitutionBranchID::bigint,'sysBaseCurrency_RefID',varBaseCurrencyID::bigint,'name', '254000000000007'::varchar,'iconSource', '97000000000029'::varchar)))::varchar;</v>
+        <v>varSQL := varSQL || (CASE WHEN (varSQL = '') THEN '' ELSE ', ' END) || (SELECT JSON_BUILD_OBJECT ('recordID', NULL::bigint,'entities', JSON_BUILD_OBJECT ('sysLoginSession_RefID', varSystemLoginSession::bigint,'sysDataAnnotation', NULL::varchar,'sysDataSetDateTimeTZ', NULL::timestamptz,'sysDataValidityStartDateTimeTZ', NULL::timestamptz,'sysDataValidityFinishDateTimeTZ', NULL::timestamptz,'sysPartitionRemovableRecordKey_RefID', NULL::bigint,'sysBranch_RefID', varInstitutionBranchID::bigint,'sysBaseCurrency_RefID',varBaseCurrencyID::bigint,'menuGroup_RefID', '254000000000007'::bigint,'menu_RefID', '97000000000029'::bigint)))::varchar;</v>
       </c>
     </row>
     <row r="31" spans="2:11" x14ac:dyDescent="0.2">
@@ -2672,7 +2672,7 @@
       </c>
       <c r="K31" s="2" t="str">
         <f t="shared" si="1"/>
-        <v>varSQL := varSQL || (CASE WHEN (varSQL = '') THEN '' ELSE ', ' END) || (SELECT JSON_BUILD_OBJECT ('recordID', NULL::bigint,'entities', JSON_BUILD_OBJECT ('sysLoginSession_RefID', varSystemLoginSession::bigint,'sysDataAnnotation', NULL::varchar,'sysDataSetDateTimeTZ', NULL::timestamptz,'sysDataValidityStartDateTimeTZ', NULL::timestamptz,'sysDataValidityFinishDateTimeTZ', NULL::timestamptz,'sysPartitionRemovableRecordKey_RefID', NULL::bigint,'sysBranch_RefID', varInstitutionBranchID::bigint,'sysBaseCurrency_RefID',varBaseCurrencyID::bigint,'name', '254000000000007'::varchar,'iconSource', '97000000000030'::varchar)))::varchar;</v>
+        <v>varSQL := varSQL || (CASE WHEN (varSQL = '') THEN '' ELSE ', ' END) || (SELECT JSON_BUILD_OBJECT ('recordID', NULL::bigint,'entities', JSON_BUILD_OBJECT ('sysLoginSession_RefID', varSystemLoginSession::bigint,'sysDataAnnotation', NULL::varchar,'sysDataSetDateTimeTZ', NULL::timestamptz,'sysDataValidityStartDateTimeTZ', NULL::timestamptz,'sysDataValidityFinishDateTimeTZ', NULL::timestamptz,'sysPartitionRemovableRecordKey_RefID', NULL::bigint,'sysBranch_RefID', varInstitutionBranchID::bigint,'sysBaseCurrency_RefID',varBaseCurrencyID::bigint,'menuGroup_RefID', '254000000000007'::bigint,'menu_RefID', '97000000000030'::bigint)))::varchar;</v>
       </c>
     </row>
     <row r="32" spans="2:11" x14ac:dyDescent="0.2">
@@ -2704,7 +2704,7 @@
       </c>
       <c r="K32" s="2" t="str">
         <f t="shared" si="1"/>
-        <v>varSQL := varSQL || (CASE WHEN (varSQL = '') THEN '' ELSE ', ' END) || (SELECT JSON_BUILD_OBJECT ('recordID', NULL::bigint,'entities', JSON_BUILD_OBJECT ('sysLoginSession_RefID', varSystemLoginSession::bigint,'sysDataAnnotation', NULL::varchar,'sysDataSetDateTimeTZ', NULL::timestamptz,'sysDataValidityStartDateTimeTZ', NULL::timestamptz,'sysDataValidityFinishDateTimeTZ', NULL::timestamptz,'sysPartitionRemovableRecordKey_RefID', NULL::bigint,'sysBranch_RefID', varInstitutionBranchID::bigint,'sysBaseCurrency_RefID',varBaseCurrencyID::bigint,'name', '254000000000007'::varchar,'iconSource', '97000000000031'::varchar)))::varchar;</v>
+        <v>varSQL := varSQL || (CASE WHEN (varSQL = '') THEN '' ELSE ', ' END) || (SELECT JSON_BUILD_OBJECT ('recordID', NULL::bigint,'entities', JSON_BUILD_OBJECT ('sysLoginSession_RefID', varSystemLoginSession::bigint,'sysDataAnnotation', NULL::varchar,'sysDataSetDateTimeTZ', NULL::timestamptz,'sysDataValidityStartDateTimeTZ', NULL::timestamptz,'sysDataValidityFinishDateTimeTZ', NULL::timestamptz,'sysPartitionRemovableRecordKey_RefID', NULL::bigint,'sysBranch_RefID', varInstitutionBranchID::bigint,'sysBaseCurrency_RefID',varBaseCurrencyID::bigint,'menuGroup_RefID', '254000000000007'::bigint,'menu_RefID', '97000000000031'::bigint)))::varchar;</v>
       </c>
     </row>
     <row r="33" spans="2:11" x14ac:dyDescent="0.2">
@@ -2736,7 +2736,7 @@
       </c>
       <c r="K33" s="2" t="str">
         <f t="shared" si="1"/>
-        <v>varSQL := varSQL || (CASE WHEN (varSQL = '') THEN '' ELSE ', ' END) || (SELECT JSON_BUILD_OBJECT ('recordID', NULL::bigint,'entities', JSON_BUILD_OBJECT ('sysLoginSession_RefID', varSystemLoginSession::bigint,'sysDataAnnotation', NULL::varchar,'sysDataSetDateTimeTZ', NULL::timestamptz,'sysDataValidityStartDateTimeTZ', NULL::timestamptz,'sysDataValidityFinishDateTimeTZ', NULL::timestamptz,'sysPartitionRemovableRecordKey_RefID', NULL::bigint,'sysBranch_RefID', varInstitutionBranchID::bigint,'sysBaseCurrency_RefID',varBaseCurrencyID::bigint,'name', '254000000000007'::varchar,'iconSource', '97000000000032'::varchar)))::varchar;</v>
+        <v>varSQL := varSQL || (CASE WHEN (varSQL = '') THEN '' ELSE ', ' END) || (SELECT JSON_BUILD_OBJECT ('recordID', NULL::bigint,'entities', JSON_BUILD_OBJECT ('sysLoginSession_RefID', varSystemLoginSession::bigint,'sysDataAnnotation', NULL::varchar,'sysDataSetDateTimeTZ', NULL::timestamptz,'sysDataValidityStartDateTimeTZ', NULL::timestamptz,'sysDataValidityFinishDateTimeTZ', NULL::timestamptz,'sysPartitionRemovableRecordKey_RefID', NULL::bigint,'sysBranch_RefID', varInstitutionBranchID::bigint,'sysBaseCurrency_RefID',varBaseCurrencyID::bigint,'menuGroup_RefID', '254000000000007'::bigint,'menu_RefID', '97000000000032'::bigint)))::varchar;</v>
       </c>
     </row>
     <row r="34" spans="2:11" x14ac:dyDescent="0.2">
@@ -2768,7 +2768,7 @@
       </c>
       <c r="K34" s="2" t="str">
         <f t="shared" si="1"/>
-        <v>varSQL := varSQL || (CASE WHEN (varSQL = '') THEN '' ELSE ', ' END) || (SELECT JSON_BUILD_OBJECT ('recordID', NULL::bigint,'entities', JSON_BUILD_OBJECT ('sysLoginSession_RefID', varSystemLoginSession::bigint,'sysDataAnnotation', NULL::varchar,'sysDataSetDateTimeTZ', NULL::timestamptz,'sysDataValidityStartDateTimeTZ', NULL::timestamptz,'sysDataValidityFinishDateTimeTZ', NULL::timestamptz,'sysPartitionRemovableRecordKey_RefID', NULL::bigint,'sysBranch_RefID', varInstitutionBranchID::bigint,'sysBaseCurrency_RefID',varBaseCurrencyID::bigint,'name', '254000000000007'::varchar,'iconSource', '97000000000033'::varchar)))::varchar;</v>
+        <v>varSQL := varSQL || (CASE WHEN (varSQL = '') THEN '' ELSE ', ' END) || (SELECT JSON_BUILD_OBJECT ('recordID', NULL::bigint,'entities', JSON_BUILD_OBJECT ('sysLoginSession_RefID', varSystemLoginSession::bigint,'sysDataAnnotation', NULL::varchar,'sysDataSetDateTimeTZ', NULL::timestamptz,'sysDataValidityStartDateTimeTZ', NULL::timestamptz,'sysDataValidityFinishDateTimeTZ', NULL::timestamptz,'sysPartitionRemovableRecordKey_RefID', NULL::bigint,'sysBranch_RefID', varInstitutionBranchID::bigint,'sysBaseCurrency_RefID',varBaseCurrencyID::bigint,'menuGroup_RefID', '254000000000007'::bigint,'menu_RefID', '97000000000033'::bigint)))::varchar;</v>
       </c>
     </row>
     <row r="35" spans="2:11" x14ac:dyDescent="0.2">
@@ -2800,7 +2800,7 @@
       </c>
       <c r="K35" s="2" t="str">
         <f t="shared" si="1"/>
-        <v>varSQL := varSQL || (CASE WHEN (varSQL = '') THEN '' ELSE ', ' END) || (SELECT JSON_BUILD_OBJECT ('recordID', NULL::bigint,'entities', JSON_BUILD_OBJECT ('sysLoginSession_RefID', varSystemLoginSession::bigint,'sysDataAnnotation', NULL::varchar,'sysDataSetDateTimeTZ', NULL::timestamptz,'sysDataValidityStartDateTimeTZ', NULL::timestamptz,'sysDataValidityFinishDateTimeTZ', NULL::timestamptz,'sysPartitionRemovableRecordKey_RefID', NULL::bigint,'sysBranch_RefID', varInstitutionBranchID::bigint,'sysBaseCurrency_RefID',varBaseCurrencyID::bigint,'name', '254000000000009'::varchar,'iconSource', '97000000000034'::varchar)))::varchar;</v>
+        <v>varSQL := varSQL || (CASE WHEN (varSQL = '') THEN '' ELSE ', ' END) || (SELECT JSON_BUILD_OBJECT ('recordID', NULL::bigint,'entities', JSON_BUILD_OBJECT ('sysLoginSession_RefID', varSystemLoginSession::bigint,'sysDataAnnotation', NULL::varchar,'sysDataSetDateTimeTZ', NULL::timestamptz,'sysDataValidityStartDateTimeTZ', NULL::timestamptz,'sysDataValidityFinishDateTimeTZ', NULL::timestamptz,'sysPartitionRemovableRecordKey_RefID', NULL::bigint,'sysBranch_RefID', varInstitutionBranchID::bigint,'sysBaseCurrency_RefID',varBaseCurrencyID::bigint,'menuGroup_RefID', '254000000000009'::bigint,'menu_RefID', '97000000000034'::bigint)))::varchar;</v>
       </c>
     </row>
     <row r="36" spans="2:11" x14ac:dyDescent="0.2">
@@ -2832,7 +2832,7 @@
       </c>
       <c r="K36" s="2" t="str">
         <f t="shared" si="1"/>
-        <v>varSQL := varSQL || (CASE WHEN (varSQL = '') THEN '' ELSE ', ' END) || (SELECT JSON_BUILD_OBJECT ('recordID', NULL::bigint,'entities', JSON_BUILD_OBJECT ('sysLoginSession_RefID', varSystemLoginSession::bigint,'sysDataAnnotation', NULL::varchar,'sysDataSetDateTimeTZ', NULL::timestamptz,'sysDataValidityStartDateTimeTZ', NULL::timestamptz,'sysDataValidityFinishDateTimeTZ', NULL::timestamptz,'sysPartitionRemovableRecordKey_RefID', NULL::bigint,'sysBranch_RefID', varInstitutionBranchID::bigint,'sysBaseCurrency_RefID',varBaseCurrencyID::bigint,'name', '254000000000009'::varchar,'iconSource', '97000000000035'::varchar)))::varchar;</v>
+        <v>varSQL := varSQL || (CASE WHEN (varSQL = '') THEN '' ELSE ', ' END) || (SELECT JSON_BUILD_OBJECT ('recordID', NULL::bigint,'entities', JSON_BUILD_OBJECT ('sysLoginSession_RefID', varSystemLoginSession::bigint,'sysDataAnnotation', NULL::varchar,'sysDataSetDateTimeTZ', NULL::timestamptz,'sysDataValidityStartDateTimeTZ', NULL::timestamptz,'sysDataValidityFinishDateTimeTZ', NULL::timestamptz,'sysPartitionRemovableRecordKey_RefID', NULL::bigint,'sysBranch_RefID', varInstitutionBranchID::bigint,'sysBaseCurrency_RefID',varBaseCurrencyID::bigint,'menuGroup_RefID', '254000000000009'::bigint,'menu_RefID', '97000000000035'::bigint)))::varchar;</v>
       </c>
     </row>
     <row r="37" spans="2:11" x14ac:dyDescent="0.2">
@@ -2864,7 +2864,7 @@
       </c>
       <c r="K37" s="2" t="str">
         <f t="shared" si="1"/>
-        <v>varSQL := varSQL || (CASE WHEN (varSQL = '') THEN '' ELSE ', ' END) || (SELECT JSON_BUILD_OBJECT ('recordID', NULL::bigint,'entities', JSON_BUILD_OBJECT ('sysLoginSession_RefID', varSystemLoginSession::bigint,'sysDataAnnotation', NULL::varchar,'sysDataSetDateTimeTZ', NULL::timestamptz,'sysDataValidityStartDateTimeTZ', NULL::timestamptz,'sysDataValidityFinishDateTimeTZ', NULL::timestamptz,'sysPartitionRemovableRecordKey_RefID', NULL::bigint,'sysBranch_RefID', varInstitutionBranchID::bigint,'sysBaseCurrency_RefID',varBaseCurrencyID::bigint,'name', '254000000000009'::varchar,'iconSource', '97000000000036'::varchar)))::varchar;</v>
+        <v>varSQL := varSQL || (CASE WHEN (varSQL = '') THEN '' ELSE ', ' END) || (SELECT JSON_BUILD_OBJECT ('recordID', NULL::bigint,'entities', JSON_BUILD_OBJECT ('sysLoginSession_RefID', varSystemLoginSession::bigint,'sysDataAnnotation', NULL::varchar,'sysDataSetDateTimeTZ', NULL::timestamptz,'sysDataValidityStartDateTimeTZ', NULL::timestamptz,'sysDataValidityFinishDateTimeTZ', NULL::timestamptz,'sysPartitionRemovableRecordKey_RefID', NULL::bigint,'sysBranch_RefID', varInstitutionBranchID::bigint,'sysBaseCurrency_RefID',varBaseCurrencyID::bigint,'menuGroup_RefID', '254000000000009'::bigint,'menu_RefID', '97000000000036'::bigint)))::varchar;</v>
       </c>
     </row>
     <row r="38" spans="2:11" x14ac:dyDescent="0.2">
@@ -2896,7 +2896,7 @@
       </c>
       <c r="K38" s="2" t="str">
         <f t="shared" si="1"/>
-        <v>varSQL := varSQL || (CASE WHEN (varSQL = '') THEN '' ELSE ', ' END) || (SELECT JSON_BUILD_OBJECT ('recordID', NULL::bigint,'entities', JSON_BUILD_OBJECT ('sysLoginSession_RefID', varSystemLoginSession::bigint,'sysDataAnnotation', NULL::varchar,'sysDataSetDateTimeTZ', NULL::timestamptz,'sysDataValidityStartDateTimeTZ', NULL::timestamptz,'sysDataValidityFinishDateTimeTZ', NULL::timestamptz,'sysPartitionRemovableRecordKey_RefID', NULL::bigint,'sysBranch_RefID', varInstitutionBranchID::bigint,'sysBaseCurrency_RefID',varBaseCurrencyID::bigint,'name', '254000000000009'::varchar,'iconSource', '97000000000037'::varchar)))::varchar;</v>
+        <v>varSQL := varSQL || (CASE WHEN (varSQL = '') THEN '' ELSE ', ' END) || (SELECT JSON_BUILD_OBJECT ('recordID', NULL::bigint,'entities', JSON_BUILD_OBJECT ('sysLoginSession_RefID', varSystemLoginSession::bigint,'sysDataAnnotation', NULL::varchar,'sysDataSetDateTimeTZ', NULL::timestamptz,'sysDataValidityStartDateTimeTZ', NULL::timestamptz,'sysDataValidityFinishDateTimeTZ', NULL::timestamptz,'sysPartitionRemovableRecordKey_RefID', NULL::bigint,'sysBranch_RefID', varInstitutionBranchID::bigint,'sysBaseCurrency_RefID',varBaseCurrencyID::bigint,'menuGroup_RefID', '254000000000009'::bigint,'menu_RefID', '97000000000037'::bigint)))::varchar;</v>
       </c>
     </row>
     <row r="39" spans="2:11" x14ac:dyDescent="0.2">
@@ -2928,7 +2928,7 @@
       </c>
       <c r="K39" s="2" t="str">
         <f t="shared" si="1"/>
-        <v>varSQL := varSQL || (CASE WHEN (varSQL = '') THEN '' ELSE ', ' END) || (SELECT JSON_BUILD_OBJECT ('recordID', NULL::bigint,'entities', JSON_BUILD_OBJECT ('sysLoginSession_RefID', varSystemLoginSession::bigint,'sysDataAnnotation', NULL::varchar,'sysDataSetDateTimeTZ', NULL::timestamptz,'sysDataValidityStartDateTimeTZ', NULL::timestamptz,'sysDataValidityFinishDateTimeTZ', NULL::timestamptz,'sysPartitionRemovableRecordKey_RefID', NULL::bigint,'sysBranch_RefID', varInstitutionBranchID::bigint,'sysBaseCurrency_RefID',varBaseCurrencyID::bigint,'name', '254000000000009'::varchar,'iconSource', '97000000000038'::varchar)))::varchar;</v>
+        <v>varSQL := varSQL || (CASE WHEN (varSQL = '') THEN '' ELSE ', ' END) || (SELECT JSON_BUILD_OBJECT ('recordID', NULL::bigint,'entities', JSON_BUILD_OBJECT ('sysLoginSession_RefID', varSystemLoginSession::bigint,'sysDataAnnotation', NULL::varchar,'sysDataSetDateTimeTZ', NULL::timestamptz,'sysDataValidityStartDateTimeTZ', NULL::timestamptz,'sysDataValidityFinishDateTimeTZ', NULL::timestamptz,'sysPartitionRemovableRecordKey_RefID', NULL::bigint,'sysBranch_RefID', varInstitutionBranchID::bigint,'sysBaseCurrency_RefID',varBaseCurrencyID::bigint,'menuGroup_RefID', '254000000000009'::bigint,'menu_RefID', '97000000000038'::bigint)))::varchar;</v>
       </c>
     </row>
     <row r="40" spans="2:11" x14ac:dyDescent="0.2">
@@ -2960,7 +2960,7 @@
       </c>
       <c r="K40" s="2" t="str">
         <f t="shared" si="1"/>
-        <v>varSQL := varSQL || (CASE WHEN (varSQL = '') THEN '' ELSE ', ' END) || (SELECT JSON_BUILD_OBJECT ('recordID', NULL::bigint,'entities', JSON_BUILD_OBJECT ('sysLoginSession_RefID', varSystemLoginSession::bigint,'sysDataAnnotation', NULL::varchar,'sysDataSetDateTimeTZ', NULL::timestamptz,'sysDataValidityStartDateTimeTZ', NULL::timestamptz,'sysDataValidityFinishDateTimeTZ', NULL::timestamptz,'sysPartitionRemovableRecordKey_RefID', NULL::bigint,'sysBranch_RefID', varInstitutionBranchID::bigint,'sysBaseCurrency_RefID',varBaseCurrencyID::bigint,'name', '254000000000009'::varchar,'iconSource', '97000000000039'::varchar)))::varchar;</v>
+        <v>varSQL := varSQL || (CASE WHEN (varSQL = '') THEN '' ELSE ', ' END) || (SELECT JSON_BUILD_OBJECT ('recordID', NULL::bigint,'entities', JSON_BUILD_OBJECT ('sysLoginSession_RefID', varSystemLoginSession::bigint,'sysDataAnnotation', NULL::varchar,'sysDataSetDateTimeTZ', NULL::timestamptz,'sysDataValidityStartDateTimeTZ', NULL::timestamptz,'sysDataValidityFinishDateTimeTZ', NULL::timestamptz,'sysPartitionRemovableRecordKey_RefID', NULL::bigint,'sysBranch_RefID', varInstitutionBranchID::bigint,'sysBaseCurrency_RefID',varBaseCurrencyID::bigint,'menuGroup_RefID', '254000000000009'::bigint,'menu_RefID', '97000000000039'::bigint)))::varchar;</v>
       </c>
     </row>
     <row r="41" spans="2:11" x14ac:dyDescent="0.2">
@@ -2992,7 +2992,7 @@
       </c>
       <c r="K41" s="2" t="str">
         <f t="shared" si="1"/>
-        <v>varSQL := varSQL || (CASE WHEN (varSQL = '') THEN '' ELSE ', ' END) || (SELECT JSON_BUILD_OBJECT ('recordID', NULL::bigint,'entities', JSON_BUILD_OBJECT ('sysLoginSession_RefID', varSystemLoginSession::bigint,'sysDataAnnotation', NULL::varchar,'sysDataSetDateTimeTZ', NULL::timestamptz,'sysDataValidityStartDateTimeTZ', NULL::timestamptz,'sysDataValidityFinishDateTimeTZ', NULL::timestamptz,'sysPartitionRemovableRecordKey_RefID', NULL::bigint,'sysBranch_RefID', varInstitutionBranchID::bigint,'sysBaseCurrency_RefID',varBaseCurrencyID::bigint,'name', '254000000000009'::varchar,'iconSource', '97000000000040'::varchar)))::varchar;</v>
+        <v>varSQL := varSQL || (CASE WHEN (varSQL = '') THEN '' ELSE ', ' END) || (SELECT JSON_BUILD_OBJECT ('recordID', NULL::bigint,'entities', JSON_BUILD_OBJECT ('sysLoginSession_RefID', varSystemLoginSession::bigint,'sysDataAnnotation', NULL::varchar,'sysDataSetDateTimeTZ', NULL::timestamptz,'sysDataValidityStartDateTimeTZ', NULL::timestamptz,'sysDataValidityFinishDateTimeTZ', NULL::timestamptz,'sysPartitionRemovableRecordKey_RefID', NULL::bigint,'sysBranch_RefID', varInstitutionBranchID::bigint,'sysBaseCurrency_RefID',varBaseCurrencyID::bigint,'menuGroup_RefID', '254000000000009'::bigint,'menu_RefID', '97000000000040'::bigint)))::varchar;</v>
       </c>
     </row>
     <row r="42" spans="2:11" x14ac:dyDescent="0.2">
@@ -3024,7 +3024,7 @@
       </c>
       <c r="K42" s="2" t="str">
         <f t="shared" si="1"/>
-        <v>varSQL := varSQL || (CASE WHEN (varSQL = '') THEN '' ELSE ', ' END) || (SELECT JSON_BUILD_OBJECT ('recordID', NULL::bigint,'entities', JSON_BUILD_OBJECT ('sysLoginSession_RefID', varSystemLoginSession::bigint,'sysDataAnnotation', NULL::varchar,'sysDataSetDateTimeTZ', NULL::timestamptz,'sysDataValidityStartDateTimeTZ', NULL::timestamptz,'sysDataValidityFinishDateTimeTZ', NULL::timestamptz,'sysPartitionRemovableRecordKey_RefID', NULL::bigint,'sysBranch_RefID', varInstitutionBranchID::bigint,'sysBaseCurrency_RefID',varBaseCurrencyID::bigint,'name', '254000000000009'::varchar,'iconSource', '97000000000041'::varchar)))::varchar;</v>
+        <v>varSQL := varSQL || (CASE WHEN (varSQL = '') THEN '' ELSE ', ' END) || (SELECT JSON_BUILD_OBJECT ('recordID', NULL::bigint,'entities', JSON_BUILD_OBJECT ('sysLoginSession_RefID', varSystemLoginSession::bigint,'sysDataAnnotation', NULL::varchar,'sysDataSetDateTimeTZ', NULL::timestamptz,'sysDataValidityStartDateTimeTZ', NULL::timestamptz,'sysDataValidityFinishDateTimeTZ', NULL::timestamptz,'sysPartitionRemovableRecordKey_RefID', NULL::bigint,'sysBranch_RefID', varInstitutionBranchID::bigint,'sysBaseCurrency_RefID',varBaseCurrencyID::bigint,'menuGroup_RefID', '254000000000009'::bigint,'menu_RefID', '97000000000041'::bigint)))::varchar;</v>
       </c>
     </row>
     <row r="43" spans="2:11" x14ac:dyDescent="0.2">
@@ -3056,7 +3056,7 @@
       </c>
       <c r="K43" s="2" t="str">
         <f t="shared" si="1"/>
-        <v>varSQL := varSQL || (CASE WHEN (varSQL = '') THEN '' ELSE ', ' END) || (SELECT JSON_BUILD_OBJECT ('recordID', NULL::bigint,'entities', JSON_BUILD_OBJECT ('sysLoginSession_RefID', varSystemLoginSession::bigint,'sysDataAnnotation', NULL::varchar,'sysDataSetDateTimeTZ', NULL::timestamptz,'sysDataValidityStartDateTimeTZ', NULL::timestamptz,'sysDataValidityFinishDateTimeTZ', NULL::timestamptz,'sysPartitionRemovableRecordKey_RefID', NULL::bigint,'sysBranch_RefID', varInstitutionBranchID::bigint,'sysBaseCurrency_RefID',varBaseCurrencyID::bigint,'name', '254000000000009'::varchar,'iconSource', '97000000000042'::varchar)))::varchar;</v>
+        <v>varSQL := varSQL || (CASE WHEN (varSQL = '') THEN '' ELSE ', ' END) || (SELECT JSON_BUILD_OBJECT ('recordID', NULL::bigint,'entities', JSON_BUILD_OBJECT ('sysLoginSession_RefID', varSystemLoginSession::bigint,'sysDataAnnotation', NULL::varchar,'sysDataSetDateTimeTZ', NULL::timestamptz,'sysDataValidityStartDateTimeTZ', NULL::timestamptz,'sysDataValidityFinishDateTimeTZ', NULL::timestamptz,'sysPartitionRemovableRecordKey_RefID', NULL::bigint,'sysBranch_RefID', varInstitutionBranchID::bigint,'sysBaseCurrency_RefID',varBaseCurrencyID::bigint,'menuGroup_RefID', '254000000000009'::bigint,'menu_RefID', '97000000000042'::bigint)))::varchar;</v>
       </c>
     </row>
     <row r="44" spans="2:11" x14ac:dyDescent="0.2">
@@ -3088,7 +3088,7 @@
       </c>
       <c r="K44" s="2" t="str">
         <f t="shared" si="1"/>
-        <v>varSQL := varSQL || (CASE WHEN (varSQL = '') THEN '' ELSE ', ' END) || (SELECT JSON_BUILD_OBJECT ('recordID', NULL::bigint,'entities', JSON_BUILD_OBJECT ('sysLoginSession_RefID', varSystemLoginSession::bigint,'sysDataAnnotation', NULL::varchar,'sysDataSetDateTimeTZ', NULL::timestamptz,'sysDataValidityStartDateTimeTZ', NULL::timestamptz,'sysDataValidityFinishDateTimeTZ', NULL::timestamptz,'sysPartitionRemovableRecordKey_RefID', NULL::bigint,'sysBranch_RefID', varInstitutionBranchID::bigint,'sysBaseCurrency_RefID',varBaseCurrencyID::bigint,'name', '254000000000009'::varchar,'iconSource', '97000000000043'::varchar)))::varchar;</v>
+        <v>varSQL := varSQL || (CASE WHEN (varSQL = '') THEN '' ELSE ', ' END) || (SELECT JSON_BUILD_OBJECT ('recordID', NULL::bigint,'entities', JSON_BUILD_OBJECT ('sysLoginSession_RefID', varSystemLoginSession::bigint,'sysDataAnnotation', NULL::varchar,'sysDataSetDateTimeTZ', NULL::timestamptz,'sysDataValidityStartDateTimeTZ', NULL::timestamptz,'sysDataValidityFinishDateTimeTZ', NULL::timestamptz,'sysPartitionRemovableRecordKey_RefID', NULL::bigint,'sysBranch_RefID', varInstitutionBranchID::bigint,'sysBaseCurrency_RefID',varBaseCurrencyID::bigint,'menuGroup_RefID', '254000000000009'::bigint,'menu_RefID', '97000000000043'::bigint)))::varchar;</v>
       </c>
     </row>
     <row r="45" spans="2:11" x14ac:dyDescent="0.2">
@@ -3120,7 +3120,7 @@
       </c>
       <c r="K45" s="2" t="str">
         <f t="shared" si="1"/>
-        <v>varSQL := varSQL || (CASE WHEN (varSQL = '') THEN '' ELSE ', ' END) || (SELECT JSON_BUILD_OBJECT ('recordID', NULL::bigint,'entities', JSON_BUILD_OBJECT ('sysLoginSession_RefID', varSystemLoginSession::bigint,'sysDataAnnotation', NULL::varchar,'sysDataSetDateTimeTZ', NULL::timestamptz,'sysDataValidityStartDateTimeTZ', NULL::timestamptz,'sysDataValidityFinishDateTimeTZ', NULL::timestamptz,'sysPartitionRemovableRecordKey_RefID', NULL::bigint,'sysBranch_RefID', varInstitutionBranchID::bigint,'sysBaseCurrency_RefID',varBaseCurrencyID::bigint,'name', '254000000000009'::varchar,'iconSource', '97000000000044'::varchar)))::varchar;</v>
+        <v>varSQL := varSQL || (CASE WHEN (varSQL = '') THEN '' ELSE ', ' END) || (SELECT JSON_BUILD_OBJECT ('recordID', NULL::bigint,'entities', JSON_BUILD_OBJECT ('sysLoginSession_RefID', varSystemLoginSession::bigint,'sysDataAnnotation', NULL::varchar,'sysDataSetDateTimeTZ', NULL::timestamptz,'sysDataValidityStartDateTimeTZ', NULL::timestamptz,'sysDataValidityFinishDateTimeTZ', NULL::timestamptz,'sysPartitionRemovableRecordKey_RefID', NULL::bigint,'sysBranch_RefID', varInstitutionBranchID::bigint,'sysBaseCurrency_RefID',varBaseCurrencyID::bigint,'menuGroup_RefID', '254000000000009'::bigint,'menu_RefID', '97000000000044'::bigint)))::varchar;</v>
       </c>
     </row>
     <row r="46" spans="2:11" x14ac:dyDescent="0.2">
@@ -3152,7 +3152,7 @@
       </c>
       <c r="K46" s="2" t="str">
         <f t="shared" si="1"/>
-        <v>varSQL := varSQL || (CASE WHEN (varSQL = '') THEN '' ELSE ', ' END) || (SELECT JSON_BUILD_OBJECT ('recordID', NULL::bigint,'entities', JSON_BUILD_OBJECT ('sysLoginSession_RefID', varSystemLoginSession::bigint,'sysDataAnnotation', NULL::varchar,'sysDataSetDateTimeTZ', NULL::timestamptz,'sysDataValidityStartDateTimeTZ', NULL::timestamptz,'sysDataValidityFinishDateTimeTZ', NULL::timestamptz,'sysPartitionRemovableRecordKey_RefID', NULL::bigint,'sysBranch_RefID', varInstitutionBranchID::bigint,'sysBaseCurrency_RefID',varBaseCurrencyID::bigint,'name', '254000000000008'::varchar,'iconSource', '97000000000045'::varchar)))::varchar;</v>
+        <v>varSQL := varSQL || (CASE WHEN (varSQL = '') THEN '' ELSE ', ' END) || (SELECT JSON_BUILD_OBJECT ('recordID', NULL::bigint,'entities', JSON_BUILD_OBJECT ('sysLoginSession_RefID', varSystemLoginSession::bigint,'sysDataAnnotation', NULL::varchar,'sysDataSetDateTimeTZ', NULL::timestamptz,'sysDataValidityStartDateTimeTZ', NULL::timestamptz,'sysDataValidityFinishDateTimeTZ', NULL::timestamptz,'sysPartitionRemovableRecordKey_RefID', NULL::bigint,'sysBranch_RefID', varInstitutionBranchID::bigint,'sysBaseCurrency_RefID',varBaseCurrencyID::bigint,'menuGroup_RefID', '254000000000008'::bigint,'menu_RefID', '97000000000045'::bigint)))::varchar;</v>
       </c>
     </row>
     <row r="47" spans="2:11" x14ac:dyDescent="0.2">
@@ -3184,7 +3184,7 @@
       </c>
       <c r="K47" s="2" t="str">
         <f t="shared" si="1"/>
-        <v>varSQL := varSQL || (CASE WHEN (varSQL = '') THEN '' ELSE ', ' END) || (SELECT JSON_BUILD_OBJECT ('recordID', NULL::bigint,'entities', JSON_BUILD_OBJECT ('sysLoginSession_RefID', varSystemLoginSession::bigint,'sysDataAnnotation', NULL::varchar,'sysDataSetDateTimeTZ', NULL::timestamptz,'sysDataValidityStartDateTimeTZ', NULL::timestamptz,'sysDataValidityFinishDateTimeTZ', NULL::timestamptz,'sysPartitionRemovableRecordKey_RefID', NULL::bigint,'sysBranch_RefID', varInstitutionBranchID::bigint,'sysBaseCurrency_RefID',varBaseCurrencyID::bigint,'name', '254000000000008'::varchar,'iconSource', '97000000000046'::varchar)))::varchar;</v>
+        <v>varSQL := varSQL || (CASE WHEN (varSQL = '') THEN '' ELSE ', ' END) || (SELECT JSON_BUILD_OBJECT ('recordID', NULL::bigint,'entities', JSON_BUILD_OBJECT ('sysLoginSession_RefID', varSystemLoginSession::bigint,'sysDataAnnotation', NULL::varchar,'sysDataSetDateTimeTZ', NULL::timestamptz,'sysDataValidityStartDateTimeTZ', NULL::timestamptz,'sysDataValidityFinishDateTimeTZ', NULL::timestamptz,'sysPartitionRemovableRecordKey_RefID', NULL::bigint,'sysBranch_RefID', varInstitutionBranchID::bigint,'sysBaseCurrency_RefID',varBaseCurrencyID::bigint,'menuGroup_RefID', '254000000000008'::bigint,'menu_RefID', '97000000000046'::bigint)))::varchar;</v>
       </c>
     </row>
     <row r="48" spans="2:11" x14ac:dyDescent="0.2">
@@ -3216,7 +3216,7 @@
       </c>
       <c r="K48" s="2" t="str">
         <f t="shared" si="1"/>
-        <v>varSQL := varSQL || (CASE WHEN (varSQL = '') THEN '' ELSE ', ' END) || (SELECT JSON_BUILD_OBJECT ('recordID', NULL::bigint,'entities', JSON_BUILD_OBJECT ('sysLoginSession_RefID', varSystemLoginSession::bigint,'sysDataAnnotation', NULL::varchar,'sysDataSetDateTimeTZ', NULL::timestamptz,'sysDataValidityStartDateTimeTZ', NULL::timestamptz,'sysDataValidityFinishDateTimeTZ', NULL::timestamptz,'sysPartitionRemovableRecordKey_RefID', NULL::bigint,'sysBranch_RefID', varInstitutionBranchID::bigint,'sysBaseCurrency_RefID',varBaseCurrencyID::bigint,'name', '254000000000008'::varchar,'iconSource', '97000000000047'::varchar)))::varchar;</v>
+        <v>varSQL := varSQL || (CASE WHEN (varSQL = '') THEN '' ELSE ', ' END) || (SELECT JSON_BUILD_OBJECT ('recordID', NULL::bigint,'entities', JSON_BUILD_OBJECT ('sysLoginSession_RefID', varSystemLoginSession::bigint,'sysDataAnnotation', NULL::varchar,'sysDataSetDateTimeTZ', NULL::timestamptz,'sysDataValidityStartDateTimeTZ', NULL::timestamptz,'sysDataValidityFinishDateTimeTZ', NULL::timestamptz,'sysPartitionRemovableRecordKey_RefID', NULL::bigint,'sysBranch_RefID', varInstitutionBranchID::bigint,'sysBaseCurrency_RefID',varBaseCurrencyID::bigint,'menuGroup_RefID', '254000000000008'::bigint,'menu_RefID', '97000000000047'::bigint)))::varchar;</v>
       </c>
     </row>
     <row r="49" spans="2:11" x14ac:dyDescent="0.2">
@@ -3248,7 +3248,7 @@
       </c>
       <c r="K49" s="2" t="str">
         <f t="shared" si="1"/>
-        <v>varSQL := varSQL || (CASE WHEN (varSQL = '') THEN '' ELSE ', ' END) || (SELECT JSON_BUILD_OBJECT ('recordID', NULL::bigint,'entities', JSON_BUILD_OBJECT ('sysLoginSession_RefID', varSystemLoginSession::bigint,'sysDataAnnotation', NULL::varchar,'sysDataSetDateTimeTZ', NULL::timestamptz,'sysDataValidityStartDateTimeTZ', NULL::timestamptz,'sysDataValidityFinishDateTimeTZ', NULL::timestamptz,'sysPartitionRemovableRecordKey_RefID', NULL::bigint,'sysBranch_RefID', varInstitutionBranchID::bigint,'sysBaseCurrency_RefID',varBaseCurrencyID::bigint,'name', '254000000000008'::varchar,'iconSource', '97000000000048'::varchar)))::varchar;</v>
+        <v>varSQL := varSQL || (CASE WHEN (varSQL = '') THEN '' ELSE ', ' END) || (SELECT JSON_BUILD_OBJECT ('recordID', NULL::bigint,'entities', JSON_BUILD_OBJECT ('sysLoginSession_RefID', varSystemLoginSession::bigint,'sysDataAnnotation', NULL::varchar,'sysDataSetDateTimeTZ', NULL::timestamptz,'sysDataValidityStartDateTimeTZ', NULL::timestamptz,'sysDataValidityFinishDateTimeTZ', NULL::timestamptz,'sysPartitionRemovableRecordKey_RefID', NULL::bigint,'sysBranch_RefID', varInstitutionBranchID::bigint,'sysBaseCurrency_RefID',varBaseCurrencyID::bigint,'menuGroup_RefID', '254000000000008'::bigint,'menu_RefID', '97000000000048'::bigint)))::varchar;</v>
       </c>
     </row>
     <row r="50" spans="2:11" x14ac:dyDescent="0.2">
@@ -3280,7 +3280,7 @@
       </c>
       <c r="K50" s="2" t="str">
         <f t="shared" si="1"/>
-        <v>varSQL := varSQL || (CASE WHEN (varSQL = '') THEN '' ELSE ', ' END) || (SELECT JSON_BUILD_OBJECT ('recordID', NULL::bigint,'entities', JSON_BUILD_OBJECT ('sysLoginSession_RefID', varSystemLoginSession::bigint,'sysDataAnnotation', NULL::varchar,'sysDataSetDateTimeTZ', NULL::timestamptz,'sysDataValidityStartDateTimeTZ', NULL::timestamptz,'sysDataValidityFinishDateTimeTZ', NULL::timestamptz,'sysPartitionRemovableRecordKey_RefID', NULL::bigint,'sysBranch_RefID', varInstitutionBranchID::bigint,'sysBaseCurrency_RefID',varBaseCurrencyID::bigint,'name', '254000000000008'::varchar,'iconSource', '97000000000049'::varchar)))::varchar;</v>
+        <v>varSQL := varSQL || (CASE WHEN (varSQL = '') THEN '' ELSE ', ' END) || (SELECT JSON_BUILD_OBJECT ('recordID', NULL::bigint,'entities', JSON_BUILD_OBJECT ('sysLoginSession_RefID', varSystemLoginSession::bigint,'sysDataAnnotation', NULL::varchar,'sysDataSetDateTimeTZ', NULL::timestamptz,'sysDataValidityStartDateTimeTZ', NULL::timestamptz,'sysDataValidityFinishDateTimeTZ', NULL::timestamptz,'sysPartitionRemovableRecordKey_RefID', NULL::bigint,'sysBranch_RefID', varInstitutionBranchID::bigint,'sysBaseCurrency_RefID',varBaseCurrencyID::bigint,'menuGroup_RefID', '254000000000008'::bigint,'menu_RefID', '97000000000049'::bigint)))::varchar;</v>
       </c>
     </row>
     <row r="51" spans="2:11" x14ac:dyDescent="0.2">
@@ -3312,7 +3312,7 @@
       </c>
       <c r="K51" s="2" t="str">
         <f t="shared" si="1"/>
-        <v>varSQL := varSQL || (CASE WHEN (varSQL = '') THEN '' ELSE ', ' END) || (SELECT JSON_BUILD_OBJECT ('recordID', NULL::bigint,'entities', JSON_BUILD_OBJECT ('sysLoginSession_RefID', varSystemLoginSession::bigint,'sysDataAnnotation', NULL::varchar,'sysDataSetDateTimeTZ', NULL::timestamptz,'sysDataValidityStartDateTimeTZ', NULL::timestamptz,'sysDataValidityFinishDateTimeTZ', NULL::timestamptz,'sysPartitionRemovableRecordKey_RefID', NULL::bigint,'sysBranch_RefID', varInstitutionBranchID::bigint,'sysBaseCurrency_RefID',varBaseCurrencyID::bigint,'name', '254000000000008'::varchar,'iconSource', '97000000000050'::varchar)))::varchar;</v>
+        <v>varSQL := varSQL || (CASE WHEN (varSQL = '') THEN '' ELSE ', ' END) || (SELECT JSON_BUILD_OBJECT ('recordID', NULL::bigint,'entities', JSON_BUILD_OBJECT ('sysLoginSession_RefID', varSystemLoginSession::bigint,'sysDataAnnotation', NULL::varchar,'sysDataSetDateTimeTZ', NULL::timestamptz,'sysDataValidityStartDateTimeTZ', NULL::timestamptz,'sysDataValidityFinishDateTimeTZ', NULL::timestamptz,'sysPartitionRemovableRecordKey_RefID', NULL::bigint,'sysBranch_RefID', varInstitutionBranchID::bigint,'sysBaseCurrency_RefID',varBaseCurrencyID::bigint,'menuGroup_RefID', '254000000000008'::bigint,'menu_RefID', '97000000000050'::bigint)))::varchar;</v>
       </c>
     </row>
     <row r="52" spans="2:11" x14ac:dyDescent="0.2">
@@ -3344,7 +3344,7 @@
       </c>
       <c r="K52" s="2" t="str">
         <f t="shared" si="1"/>
-        <v>varSQL := varSQL || (CASE WHEN (varSQL = '') THEN '' ELSE ', ' END) || (SELECT JSON_BUILD_OBJECT ('recordID', NULL::bigint,'entities', JSON_BUILD_OBJECT ('sysLoginSession_RefID', varSystemLoginSession::bigint,'sysDataAnnotation', NULL::varchar,'sysDataSetDateTimeTZ', NULL::timestamptz,'sysDataValidityStartDateTimeTZ', NULL::timestamptz,'sysDataValidityFinishDateTimeTZ', NULL::timestamptz,'sysPartitionRemovableRecordKey_RefID', NULL::bigint,'sysBranch_RefID', varInstitutionBranchID::bigint,'sysBaseCurrency_RefID',varBaseCurrencyID::bigint,'name', '254000000000008'::varchar,'iconSource', '97000000000051'::varchar)))::varchar;</v>
+        <v>varSQL := varSQL || (CASE WHEN (varSQL = '') THEN '' ELSE ', ' END) || (SELECT JSON_BUILD_OBJECT ('recordID', NULL::bigint,'entities', JSON_BUILD_OBJECT ('sysLoginSession_RefID', varSystemLoginSession::bigint,'sysDataAnnotation', NULL::varchar,'sysDataSetDateTimeTZ', NULL::timestamptz,'sysDataValidityStartDateTimeTZ', NULL::timestamptz,'sysDataValidityFinishDateTimeTZ', NULL::timestamptz,'sysPartitionRemovableRecordKey_RefID', NULL::bigint,'sysBranch_RefID', varInstitutionBranchID::bigint,'sysBaseCurrency_RefID',varBaseCurrencyID::bigint,'menuGroup_RefID', '254000000000008'::bigint,'menu_RefID', '97000000000051'::bigint)))::varchar;</v>
       </c>
     </row>
     <row r="53" spans="2:11" x14ac:dyDescent="0.2">
@@ -3376,7 +3376,7 @@
       </c>
       <c r="K53" s="2" t="str">
         <f t="shared" si="1"/>
-        <v>varSQL := varSQL || (CASE WHEN (varSQL = '') THEN '' ELSE ', ' END) || (SELECT JSON_BUILD_OBJECT ('recordID', NULL::bigint,'entities', JSON_BUILD_OBJECT ('sysLoginSession_RefID', varSystemLoginSession::bigint,'sysDataAnnotation', NULL::varchar,'sysDataSetDateTimeTZ', NULL::timestamptz,'sysDataValidityStartDateTimeTZ', NULL::timestamptz,'sysDataValidityFinishDateTimeTZ', NULL::timestamptz,'sysPartitionRemovableRecordKey_RefID', NULL::bigint,'sysBranch_RefID', varInstitutionBranchID::bigint,'sysBaseCurrency_RefID',varBaseCurrencyID::bigint,'name', '254000000000008'::varchar,'iconSource', '97000000000052'::varchar)))::varchar;</v>
+        <v>varSQL := varSQL || (CASE WHEN (varSQL = '') THEN '' ELSE ', ' END) || (SELECT JSON_BUILD_OBJECT ('recordID', NULL::bigint,'entities', JSON_BUILD_OBJECT ('sysLoginSession_RefID', varSystemLoginSession::bigint,'sysDataAnnotation', NULL::varchar,'sysDataSetDateTimeTZ', NULL::timestamptz,'sysDataValidityStartDateTimeTZ', NULL::timestamptz,'sysDataValidityFinishDateTimeTZ', NULL::timestamptz,'sysPartitionRemovableRecordKey_RefID', NULL::bigint,'sysBranch_RefID', varInstitutionBranchID::bigint,'sysBaseCurrency_RefID',varBaseCurrencyID::bigint,'menuGroup_RefID', '254000000000008'::bigint,'menu_RefID', '97000000000052'::bigint)))::varchar;</v>
       </c>
     </row>
     <row r="54" spans="2:11" x14ac:dyDescent="0.2">
@@ -3408,7 +3408,7 @@
       </c>
       <c r="K54" s="2" t="str">
         <f t="shared" si="1"/>
-        <v>varSQL := varSQL || (CASE WHEN (varSQL = '') THEN '' ELSE ', ' END) || (SELECT JSON_BUILD_OBJECT ('recordID', NULL::bigint,'entities', JSON_BUILD_OBJECT ('sysLoginSession_RefID', varSystemLoginSession::bigint,'sysDataAnnotation', NULL::varchar,'sysDataSetDateTimeTZ', NULL::timestamptz,'sysDataValidityStartDateTimeTZ', NULL::timestamptz,'sysDataValidityFinishDateTimeTZ', NULL::timestamptz,'sysPartitionRemovableRecordKey_RefID', NULL::bigint,'sysBranch_RefID', varInstitutionBranchID::bigint,'sysBaseCurrency_RefID',varBaseCurrencyID::bigint,'name', '254000000000008'::varchar,'iconSource', '97000000000053'::varchar)))::varchar;</v>
+        <v>varSQL := varSQL || (CASE WHEN (varSQL = '') THEN '' ELSE ', ' END) || (SELECT JSON_BUILD_OBJECT ('recordID', NULL::bigint,'entities', JSON_BUILD_OBJECT ('sysLoginSession_RefID', varSystemLoginSession::bigint,'sysDataAnnotation', NULL::varchar,'sysDataSetDateTimeTZ', NULL::timestamptz,'sysDataValidityStartDateTimeTZ', NULL::timestamptz,'sysDataValidityFinishDateTimeTZ', NULL::timestamptz,'sysPartitionRemovableRecordKey_RefID', NULL::bigint,'sysBranch_RefID', varInstitutionBranchID::bigint,'sysBaseCurrency_RefID',varBaseCurrencyID::bigint,'menuGroup_RefID', '254000000000008'::bigint,'menu_RefID', '97000000000053'::bigint)))::varchar;</v>
       </c>
     </row>
     <row r="55" spans="2:11" x14ac:dyDescent="0.2">
@@ -3440,7 +3440,7 @@
       </c>
       <c r="K55" s="2" t="str">
         <f t="shared" si="1"/>
-        <v>varSQL := varSQL || (CASE WHEN (varSQL = '') THEN '' ELSE ', ' END) || (SELECT JSON_BUILD_OBJECT ('recordID', NULL::bigint,'entities', JSON_BUILD_OBJECT ('sysLoginSession_RefID', varSystemLoginSession::bigint,'sysDataAnnotation', NULL::varchar,'sysDataSetDateTimeTZ', NULL::timestamptz,'sysDataValidityStartDateTimeTZ', NULL::timestamptz,'sysDataValidityFinishDateTimeTZ', NULL::timestamptz,'sysPartitionRemovableRecordKey_RefID', NULL::bigint,'sysBranch_RefID', varInstitutionBranchID::bigint,'sysBaseCurrency_RefID',varBaseCurrencyID::bigint,'name', '254000000000008'::varchar,'iconSource', '97000000000054'::varchar)))::varchar;</v>
+        <v>varSQL := varSQL || (CASE WHEN (varSQL = '') THEN '' ELSE ', ' END) || (SELECT JSON_BUILD_OBJECT ('recordID', NULL::bigint,'entities', JSON_BUILD_OBJECT ('sysLoginSession_RefID', varSystemLoginSession::bigint,'sysDataAnnotation', NULL::varchar,'sysDataSetDateTimeTZ', NULL::timestamptz,'sysDataValidityStartDateTimeTZ', NULL::timestamptz,'sysDataValidityFinishDateTimeTZ', NULL::timestamptz,'sysPartitionRemovableRecordKey_RefID', NULL::bigint,'sysBranch_RefID', varInstitutionBranchID::bigint,'sysBaseCurrency_RefID',varBaseCurrencyID::bigint,'menuGroup_RefID', '254000000000008'::bigint,'menu_RefID', '97000000000054'::bigint)))::varchar;</v>
       </c>
     </row>
     <row r="56" spans="2:11" x14ac:dyDescent="0.2">
@@ -3472,7 +3472,7 @@
       </c>
       <c r="K56" s="2" t="str">
         <f t="shared" si="1"/>
-        <v>varSQL := varSQL || (CASE WHEN (varSQL = '') THEN '' ELSE ', ' END) || (SELECT JSON_BUILD_OBJECT ('recordID', NULL::bigint,'entities', JSON_BUILD_OBJECT ('sysLoginSession_RefID', varSystemLoginSession::bigint,'sysDataAnnotation', NULL::varchar,'sysDataSetDateTimeTZ', NULL::timestamptz,'sysDataValidityStartDateTimeTZ', NULL::timestamptz,'sysDataValidityFinishDateTimeTZ', NULL::timestamptz,'sysPartitionRemovableRecordKey_RefID', NULL::bigint,'sysBranch_RefID', varInstitutionBranchID::bigint,'sysBaseCurrency_RefID',varBaseCurrencyID::bigint,'name', '254000000000010'::varchar,'iconSource', '97000000000055'::varchar)))::varchar;</v>
+        <v>varSQL := varSQL || (CASE WHEN (varSQL = '') THEN '' ELSE ', ' END) || (SELECT JSON_BUILD_OBJECT ('recordID', NULL::bigint,'entities', JSON_BUILD_OBJECT ('sysLoginSession_RefID', varSystemLoginSession::bigint,'sysDataAnnotation', NULL::varchar,'sysDataSetDateTimeTZ', NULL::timestamptz,'sysDataValidityStartDateTimeTZ', NULL::timestamptz,'sysDataValidityFinishDateTimeTZ', NULL::timestamptz,'sysPartitionRemovableRecordKey_RefID', NULL::bigint,'sysBranch_RefID', varInstitutionBranchID::bigint,'sysBaseCurrency_RefID',varBaseCurrencyID::bigint,'menuGroup_RefID', '254000000000010'::bigint,'menu_RefID', '97000000000055'::bigint)))::varchar;</v>
       </c>
     </row>
     <row r="57" spans="2:11" x14ac:dyDescent="0.2">
@@ -3504,7 +3504,7 @@
       </c>
       <c r="K57" s="2" t="str">
         <f t="shared" si="1"/>
-        <v>varSQL := varSQL || (CASE WHEN (varSQL = '') THEN '' ELSE ', ' END) || (SELECT JSON_BUILD_OBJECT ('recordID', NULL::bigint,'entities', JSON_BUILD_OBJECT ('sysLoginSession_RefID', varSystemLoginSession::bigint,'sysDataAnnotation', NULL::varchar,'sysDataSetDateTimeTZ', NULL::timestamptz,'sysDataValidityStartDateTimeTZ', NULL::timestamptz,'sysDataValidityFinishDateTimeTZ', NULL::timestamptz,'sysPartitionRemovableRecordKey_RefID', NULL::bigint,'sysBranch_RefID', varInstitutionBranchID::bigint,'sysBaseCurrency_RefID',varBaseCurrencyID::bigint,'name', '254000000000010'::varchar,'iconSource', '97000000000056'::varchar)))::varchar;</v>
+        <v>varSQL := varSQL || (CASE WHEN (varSQL = '') THEN '' ELSE ', ' END) || (SELECT JSON_BUILD_OBJECT ('recordID', NULL::bigint,'entities', JSON_BUILD_OBJECT ('sysLoginSession_RefID', varSystemLoginSession::bigint,'sysDataAnnotation', NULL::varchar,'sysDataSetDateTimeTZ', NULL::timestamptz,'sysDataValidityStartDateTimeTZ', NULL::timestamptz,'sysDataValidityFinishDateTimeTZ', NULL::timestamptz,'sysPartitionRemovableRecordKey_RefID', NULL::bigint,'sysBranch_RefID', varInstitutionBranchID::bigint,'sysBaseCurrency_RefID',varBaseCurrencyID::bigint,'menuGroup_RefID', '254000000000010'::bigint,'menu_RefID', '97000000000056'::bigint)))::varchar;</v>
       </c>
     </row>
     <row r="58" spans="2:11" x14ac:dyDescent="0.2">
@@ -3536,7 +3536,7 @@
       </c>
       <c r="K58" s="2" t="str">
         <f t="shared" si="1"/>
-        <v>varSQL := varSQL || (CASE WHEN (varSQL = '') THEN '' ELSE ', ' END) || (SELECT JSON_BUILD_OBJECT ('recordID', NULL::bigint,'entities', JSON_BUILD_OBJECT ('sysLoginSession_RefID', varSystemLoginSession::bigint,'sysDataAnnotation', NULL::varchar,'sysDataSetDateTimeTZ', NULL::timestamptz,'sysDataValidityStartDateTimeTZ', NULL::timestamptz,'sysDataValidityFinishDateTimeTZ', NULL::timestamptz,'sysPartitionRemovableRecordKey_RefID', NULL::bigint,'sysBranch_RefID', varInstitutionBranchID::bigint,'sysBaseCurrency_RefID',varBaseCurrencyID::bigint,'name', '254000000000010'::varchar,'iconSource', '97000000000057'::varchar)))::varchar;</v>
+        <v>varSQL := varSQL || (CASE WHEN (varSQL = '') THEN '' ELSE ', ' END) || (SELECT JSON_BUILD_OBJECT ('recordID', NULL::bigint,'entities', JSON_BUILD_OBJECT ('sysLoginSession_RefID', varSystemLoginSession::bigint,'sysDataAnnotation', NULL::varchar,'sysDataSetDateTimeTZ', NULL::timestamptz,'sysDataValidityStartDateTimeTZ', NULL::timestamptz,'sysDataValidityFinishDateTimeTZ', NULL::timestamptz,'sysPartitionRemovableRecordKey_RefID', NULL::bigint,'sysBranch_RefID', varInstitutionBranchID::bigint,'sysBaseCurrency_RefID',varBaseCurrencyID::bigint,'menuGroup_RefID', '254000000000010'::bigint,'menu_RefID', '97000000000057'::bigint)))::varchar;</v>
       </c>
     </row>
     <row r="59" spans="2:11" x14ac:dyDescent="0.2">
@@ -3568,7 +3568,7 @@
       </c>
       <c r="K59" s="2" t="str">
         <f t="shared" si="1"/>
-        <v>varSQL := varSQL || (CASE WHEN (varSQL = '') THEN '' ELSE ', ' END) || (SELECT JSON_BUILD_OBJECT ('recordID', NULL::bigint,'entities', JSON_BUILD_OBJECT ('sysLoginSession_RefID', varSystemLoginSession::bigint,'sysDataAnnotation', NULL::varchar,'sysDataSetDateTimeTZ', NULL::timestamptz,'sysDataValidityStartDateTimeTZ', NULL::timestamptz,'sysDataValidityFinishDateTimeTZ', NULL::timestamptz,'sysPartitionRemovableRecordKey_RefID', NULL::bigint,'sysBranch_RefID', varInstitutionBranchID::bigint,'sysBaseCurrency_RefID',varBaseCurrencyID::bigint,'name', '254000000000010'::varchar,'iconSource', '97000000000058'::varchar)))::varchar;</v>
+        <v>varSQL := varSQL || (CASE WHEN (varSQL = '') THEN '' ELSE ', ' END) || (SELECT JSON_BUILD_OBJECT ('recordID', NULL::bigint,'entities', JSON_BUILD_OBJECT ('sysLoginSession_RefID', varSystemLoginSession::bigint,'sysDataAnnotation', NULL::varchar,'sysDataSetDateTimeTZ', NULL::timestamptz,'sysDataValidityStartDateTimeTZ', NULL::timestamptz,'sysDataValidityFinishDateTimeTZ', NULL::timestamptz,'sysPartitionRemovableRecordKey_RefID', NULL::bigint,'sysBranch_RefID', varInstitutionBranchID::bigint,'sysBaseCurrency_RefID',varBaseCurrencyID::bigint,'menuGroup_RefID', '254000000000010'::bigint,'menu_RefID', '97000000000058'::bigint)))::varchar;</v>
       </c>
     </row>
     <row r="60" spans="2:11" x14ac:dyDescent="0.2">
@@ -3600,7 +3600,7 @@
       </c>
       <c r="K60" s="2" t="str">
         <f t="shared" si="1"/>
-        <v>varSQL := varSQL || (CASE WHEN (varSQL = '') THEN '' ELSE ', ' END) || (SELECT JSON_BUILD_OBJECT ('recordID', NULL::bigint,'entities', JSON_BUILD_OBJECT ('sysLoginSession_RefID', varSystemLoginSession::bigint,'sysDataAnnotation', NULL::varchar,'sysDataSetDateTimeTZ', NULL::timestamptz,'sysDataValidityStartDateTimeTZ', NULL::timestamptz,'sysDataValidityFinishDateTimeTZ', NULL::timestamptz,'sysPartitionRemovableRecordKey_RefID', NULL::bigint,'sysBranch_RefID', varInstitutionBranchID::bigint,'sysBaseCurrency_RefID',varBaseCurrencyID::bigint,'name', '254000000000010'::varchar,'iconSource', '97000000000059'::varchar)))::varchar;</v>
+        <v>varSQL := varSQL || (CASE WHEN (varSQL = '') THEN '' ELSE ', ' END) || (SELECT JSON_BUILD_OBJECT ('recordID', NULL::bigint,'entities', JSON_BUILD_OBJECT ('sysLoginSession_RefID', varSystemLoginSession::bigint,'sysDataAnnotation', NULL::varchar,'sysDataSetDateTimeTZ', NULL::timestamptz,'sysDataValidityStartDateTimeTZ', NULL::timestamptz,'sysDataValidityFinishDateTimeTZ', NULL::timestamptz,'sysPartitionRemovableRecordKey_RefID', NULL::bigint,'sysBranch_RefID', varInstitutionBranchID::bigint,'sysBaseCurrency_RefID',varBaseCurrencyID::bigint,'menuGroup_RefID', '254000000000010'::bigint,'menu_RefID', '97000000000059'::bigint)))::varchar;</v>
       </c>
     </row>
     <row r="61" spans="2:11" x14ac:dyDescent="0.2">
@@ -3632,7 +3632,7 @@
       </c>
       <c r="K61" s="2" t="str">
         <f t="shared" si="1"/>
-        <v>varSQL := varSQL || (CASE WHEN (varSQL = '') THEN '' ELSE ', ' END) || (SELECT JSON_BUILD_OBJECT ('recordID', NULL::bigint,'entities', JSON_BUILD_OBJECT ('sysLoginSession_RefID', varSystemLoginSession::bigint,'sysDataAnnotation', NULL::varchar,'sysDataSetDateTimeTZ', NULL::timestamptz,'sysDataValidityStartDateTimeTZ', NULL::timestamptz,'sysDataValidityFinishDateTimeTZ', NULL::timestamptz,'sysPartitionRemovableRecordKey_RefID', NULL::bigint,'sysBranch_RefID', varInstitutionBranchID::bigint,'sysBaseCurrency_RefID',varBaseCurrencyID::bigint,'name', '254000000000010'::varchar,'iconSource', '97000000000060'::varchar)))::varchar;</v>
+        <v>varSQL := varSQL || (CASE WHEN (varSQL = '') THEN '' ELSE ', ' END) || (SELECT JSON_BUILD_OBJECT ('recordID', NULL::bigint,'entities', JSON_BUILD_OBJECT ('sysLoginSession_RefID', varSystemLoginSession::bigint,'sysDataAnnotation', NULL::varchar,'sysDataSetDateTimeTZ', NULL::timestamptz,'sysDataValidityStartDateTimeTZ', NULL::timestamptz,'sysDataValidityFinishDateTimeTZ', NULL::timestamptz,'sysPartitionRemovableRecordKey_RefID', NULL::bigint,'sysBranch_RefID', varInstitutionBranchID::bigint,'sysBaseCurrency_RefID',varBaseCurrencyID::bigint,'menuGroup_RefID', '254000000000010'::bigint,'menu_RefID', '97000000000060'::bigint)))::varchar;</v>
       </c>
     </row>
     <row r="62" spans="2:11" x14ac:dyDescent="0.2">
@@ -3664,7 +3664,7 @@
       </c>
       <c r="K62" s="2" t="str">
         <f t="shared" si="1"/>
-        <v>varSQL := varSQL || (CASE WHEN (varSQL = '') THEN '' ELSE ', ' END) || (SELECT JSON_BUILD_OBJECT ('recordID', NULL::bigint,'entities', JSON_BUILD_OBJECT ('sysLoginSession_RefID', varSystemLoginSession::bigint,'sysDataAnnotation', NULL::varchar,'sysDataSetDateTimeTZ', NULL::timestamptz,'sysDataValidityStartDateTimeTZ', NULL::timestamptz,'sysDataValidityFinishDateTimeTZ', NULL::timestamptz,'sysPartitionRemovableRecordKey_RefID', NULL::bigint,'sysBranch_RefID', varInstitutionBranchID::bigint,'sysBaseCurrency_RefID',varBaseCurrencyID::bigint,'name', '254000000000010'::varchar,'iconSource', '97000000000061'::varchar)))::varchar;</v>
+        <v>varSQL := varSQL || (CASE WHEN (varSQL = '') THEN '' ELSE ', ' END) || (SELECT JSON_BUILD_OBJECT ('recordID', NULL::bigint,'entities', JSON_BUILD_OBJECT ('sysLoginSession_RefID', varSystemLoginSession::bigint,'sysDataAnnotation', NULL::varchar,'sysDataSetDateTimeTZ', NULL::timestamptz,'sysDataValidityStartDateTimeTZ', NULL::timestamptz,'sysDataValidityFinishDateTimeTZ', NULL::timestamptz,'sysPartitionRemovableRecordKey_RefID', NULL::bigint,'sysBranch_RefID', varInstitutionBranchID::bigint,'sysBaseCurrency_RefID',varBaseCurrencyID::bigint,'menuGroup_RefID', '254000000000010'::bigint,'menu_RefID', '97000000000061'::bigint)))::varchar;</v>
       </c>
     </row>
     <row r="63" spans="2:11" x14ac:dyDescent="0.2">
@@ -3696,7 +3696,7 @@
       </c>
       <c r="K63" s="2" t="str">
         <f t="shared" si="1"/>
-        <v>varSQL := varSQL || (CASE WHEN (varSQL = '') THEN '' ELSE ', ' END) || (SELECT JSON_BUILD_OBJECT ('recordID', NULL::bigint,'entities', JSON_BUILD_OBJECT ('sysLoginSession_RefID', varSystemLoginSession::bigint,'sysDataAnnotation', NULL::varchar,'sysDataSetDateTimeTZ', NULL::timestamptz,'sysDataValidityStartDateTimeTZ', NULL::timestamptz,'sysDataValidityFinishDateTimeTZ', NULL::timestamptz,'sysPartitionRemovableRecordKey_RefID', NULL::bigint,'sysBranch_RefID', varInstitutionBranchID::bigint,'sysBaseCurrency_RefID',varBaseCurrencyID::bigint,'name', '254000000000006'::varchar,'iconSource', '97000000000062'::varchar)))::varchar;</v>
+        <v>varSQL := varSQL || (CASE WHEN (varSQL = '') THEN '' ELSE ', ' END) || (SELECT JSON_BUILD_OBJECT ('recordID', NULL::bigint,'entities', JSON_BUILD_OBJECT ('sysLoginSession_RefID', varSystemLoginSession::bigint,'sysDataAnnotation', NULL::varchar,'sysDataSetDateTimeTZ', NULL::timestamptz,'sysDataValidityStartDateTimeTZ', NULL::timestamptz,'sysDataValidityFinishDateTimeTZ', NULL::timestamptz,'sysPartitionRemovableRecordKey_RefID', NULL::bigint,'sysBranch_RefID', varInstitutionBranchID::bigint,'sysBaseCurrency_RefID',varBaseCurrencyID::bigint,'menuGroup_RefID', '254000000000006'::bigint,'menu_RefID', '97000000000062'::bigint)))::varchar;</v>
       </c>
     </row>
     <row r="64" spans="2:11" x14ac:dyDescent="0.2">
@@ -3728,7 +3728,7 @@
       </c>
       <c r="K64" s="2" t="str">
         <f t="shared" si="1"/>
-        <v>varSQL := varSQL || (CASE WHEN (varSQL = '') THEN '' ELSE ', ' END) || (SELECT JSON_BUILD_OBJECT ('recordID', NULL::bigint,'entities', JSON_BUILD_OBJECT ('sysLoginSession_RefID', varSystemLoginSession::bigint,'sysDataAnnotation', NULL::varchar,'sysDataSetDateTimeTZ', NULL::timestamptz,'sysDataValidityStartDateTimeTZ', NULL::timestamptz,'sysDataValidityFinishDateTimeTZ', NULL::timestamptz,'sysPartitionRemovableRecordKey_RefID', NULL::bigint,'sysBranch_RefID', varInstitutionBranchID::bigint,'sysBaseCurrency_RefID',varBaseCurrencyID::bigint,'name', '254000000000006'::varchar,'iconSource', '97000000000063'::varchar)))::varchar;</v>
+        <v>varSQL := varSQL || (CASE WHEN (varSQL = '') THEN '' ELSE ', ' END) || (SELECT JSON_BUILD_OBJECT ('recordID', NULL::bigint,'entities', JSON_BUILD_OBJECT ('sysLoginSession_RefID', varSystemLoginSession::bigint,'sysDataAnnotation', NULL::varchar,'sysDataSetDateTimeTZ', NULL::timestamptz,'sysDataValidityStartDateTimeTZ', NULL::timestamptz,'sysDataValidityFinishDateTimeTZ', NULL::timestamptz,'sysPartitionRemovableRecordKey_RefID', NULL::bigint,'sysBranch_RefID', varInstitutionBranchID::bigint,'sysBaseCurrency_RefID',varBaseCurrencyID::bigint,'menuGroup_RefID', '254000000000006'::bigint,'menu_RefID', '97000000000063'::bigint)))::varchar;</v>
       </c>
     </row>
     <row r="65" spans="2:11" x14ac:dyDescent="0.2">
@@ -3760,7 +3760,7 @@
       </c>
       <c r="K65" s="2" t="str">
         <f t="shared" si="1"/>
-        <v>varSQL := varSQL || (CASE WHEN (varSQL = '') THEN '' ELSE ', ' END) || (SELECT JSON_BUILD_OBJECT ('recordID', NULL::bigint,'entities', JSON_BUILD_OBJECT ('sysLoginSession_RefID', varSystemLoginSession::bigint,'sysDataAnnotation', NULL::varchar,'sysDataSetDateTimeTZ', NULL::timestamptz,'sysDataValidityStartDateTimeTZ', NULL::timestamptz,'sysDataValidityFinishDateTimeTZ', NULL::timestamptz,'sysPartitionRemovableRecordKey_RefID', NULL::bigint,'sysBranch_RefID', varInstitutionBranchID::bigint,'sysBaseCurrency_RefID',varBaseCurrencyID::bigint,'name', '254000000000006'::varchar,'iconSource', '97000000000064'::varchar)))::varchar;</v>
+        <v>varSQL := varSQL || (CASE WHEN (varSQL = '') THEN '' ELSE ', ' END) || (SELECT JSON_BUILD_OBJECT ('recordID', NULL::bigint,'entities', JSON_BUILD_OBJECT ('sysLoginSession_RefID', varSystemLoginSession::bigint,'sysDataAnnotation', NULL::varchar,'sysDataSetDateTimeTZ', NULL::timestamptz,'sysDataValidityStartDateTimeTZ', NULL::timestamptz,'sysDataValidityFinishDateTimeTZ', NULL::timestamptz,'sysPartitionRemovableRecordKey_RefID', NULL::bigint,'sysBranch_RefID', varInstitutionBranchID::bigint,'sysBaseCurrency_RefID',varBaseCurrencyID::bigint,'menuGroup_RefID', '254000000000006'::bigint,'menu_RefID', '97000000000064'::bigint)))::varchar;</v>
       </c>
     </row>
     <row r="66" spans="2:11" x14ac:dyDescent="0.2">
@@ -3792,7 +3792,7 @@
       </c>
       <c r="K66" s="2" t="str">
         <f t="shared" si="1"/>
-        <v>varSQL := varSQL || (CASE WHEN (varSQL = '') THEN '' ELSE ', ' END) || (SELECT JSON_BUILD_OBJECT ('recordID', NULL::bigint,'entities', JSON_BUILD_OBJECT ('sysLoginSession_RefID', varSystemLoginSession::bigint,'sysDataAnnotation', NULL::varchar,'sysDataSetDateTimeTZ', NULL::timestamptz,'sysDataValidityStartDateTimeTZ', NULL::timestamptz,'sysDataValidityFinishDateTimeTZ', NULL::timestamptz,'sysPartitionRemovableRecordKey_RefID', NULL::bigint,'sysBranch_RefID', varInstitutionBranchID::bigint,'sysBaseCurrency_RefID',varBaseCurrencyID::bigint,'name', '254000000000006'::varchar,'iconSource', '97000000000065'::varchar)))::varchar;</v>
+        <v>varSQL := varSQL || (CASE WHEN (varSQL = '') THEN '' ELSE ', ' END) || (SELECT JSON_BUILD_OBJECT ('recordID', NULL::bigint,'entities', JSON_BUILD_OBJECT ('sysLoginSession_RefID', varSystemLoginSession::bigint,'sysDataAnnotation', NULL::varchar,'sysDataSetDateTimeTZ', NULL::timestamptz,'sysDataValidityStartDateTimeTZ', NULL::timestamptz,'sysDataValidityFinishDateTimeTZ', NULL::timestamptz,'sysPartitionRemovableRecordKey_RefID', NULL::bigint,'sysBranch_RefID', varInstitutionBranchID::bigint,'sysBaseCurrency_RefID',varBaseCurrencyID::bigint,'menuGroup_RefID', '254000000000006'::bigint,'menu_RefID', '97000000000065'::bigint)))::varchar;</v>
       </c>
     </row>
     <row r="67" spans="2:11" x14ac:dyDescent="0.2">
@@ -3834,10 +3834,10 @@
 "'sysPartitionRemovableRecordKey_RefID', NULL::bigint,",
 "'sysBranch_RefID', varInstitutionBranchID::bigint,",
 "'sysBaseCurrency_RefID',varBaseCurrencyID::bigint,",
-"'name', ", IF(EXACT($G67, ""), "null", CONCATENATE("'", SUBSTITUTE($G67, "'", "\'"), "'")), "::varchar,",
-"'iconSource', ", IF(EXACT($B67, ""), "null", CONCATENATE("'", SUBSTITUTE($B67, "'", "\'"), "'")), "::varchar",
+"'menuGroup_RefID', ", IF(EXACT($G67, ""), "null", CONCATENATE("'", SUBSTITUTE($G67, "'", "\'"), "'")), "::bigint,",
+"'menu_RefID', ", IF(EXACT($B67, ""), "null", CONCATENATE("'", SUBSTITUTE($B67, "'", "\'"), "'")), "::bigint",
 ")))::varchar;")</f>
-        <v>varSQL := varSQL || (CASE WHEN (varSQL = '') THEN '' ELSE ', ' END) || (SELECT JSON_BUILD_OBJECT ('recordID', NULL::bigint,'entities', JSON_BUILD_OBJECT ('sysLoginSession_RefID', varSystemLoginSession::bigint,'sysDataAnnotation', NULL::varchar,'sysDataSetDateTimeTZ', NULL::timestamptz,'sysDataValidityStartDateTimeTZ', NULL::timestamptz,'sysDataValidityFinishDateTimeTZ', NULL::timestamptz,'sysPartitionRemovableRecordKey_RefID', NULL::bigint,'sysBranch_RefID', varInstitutionBranchID::bigint,'sysBaseCurrency_RefID',varBaseCurrencyID::bigint,'name', '254000000000006'::varchar,'iconSource', '97000000000066'::varchar)))::varchar;</v>
+        <v>varSQL := varSQL || (CASE WHEN (varSQL = '') THEN '' ELSE ', ' END) || (SELECT JSON_BUILD_OBJECT ('recordID', NULL::bigint,'entities', JSON_BUILD_OBJECT ('sysLoginSession_RefID', varSystemLoginSession::bigint,'sysDataAnnotation', NULL::varchar,'sysDataSetDateTimeTZ', NULL::timestamptz,'sysDataValidityStartDateTimeTZ', NULL::timestamptz,'sysDataValidityFinishDateTimeTZ', NULL::timestamptz,'sysPartitionRemovableRecordKey_RefID', NULL::bigint,'sysBranch_RefID', varInstitutionBranchID::bigint,'sysBaseCurrency_RefID',varBaseCurrencyID::bigint,'menuGroup_RefID', '254000000000006'::bigint,'menu_RefID', '97000000000066'::bigint)))::varchar;</v>
       </c>
     </row>
     <row r="68" spans="2:11" x14ac:dyDescent="0.2">
@@ -3869,7 +3869,7 @@
       </c>
       <c r="K68" s="2" t="str">
         <f t="shared" si="3"/>
-        <v>varSQL := varSQL || (CASE WHEN (varSQL = '') THEN '' ELSE ', ' END) || (SELECT JSON_BUILD_OBJECT ('recordID', NULL::bigint,'entities', JSON_BUILD_OBJECT ('sysLoginSession_RefID', varSystemLoginSession::bigint,'sysDataAnnotation', NULL::varchar,'sysDataSetDateTimeTZ', NULL::timestamptz,'sysDataValidityStartDateTimeTZ', NULL::timestamptz,'sysDataValidityFinishDateTimeTZ', NULL::timestamptz,'sysPartitionRemovableRecordKey_RefID', NULL::bigint,'sysBranch_RefID', varInstitutionBranchID::bigint,'sysBaseCurrency_RefID',varBaseCurrencyID::bigint,'name', '254000000000006'::varchar,'iconSource', '97000000000067'::varchar)))::varchar;</v>
+        <v>varSQL := varSQL || (CASE WHEN (varSQL = '') THEN '' ELSE ', ' END) || (SELECT JSON_BUILD_OBJECT ('recordID', NULL::bigint,'entities', JSON_BUILD_OBJECT ('sysLoginSession_RefID', varSystemLoginSession::bigint,'sysDataAnnotation', NULL::varchar,'sysDataSetDateTimeTZ', NULL::timestamptz,'sysDataValidityStartDateTimeTZ', NULL::timestamptz,'sysDataValidityFinishDateTimeTZ', NULL::timestamptz,'sysPartitionRemovableRecordKey_RefID', NULL::bigint,'sysBranch_RefID', varInstitutionBranchID::bigint,'sysBaseCurrency_RefID',varBaseCurrencyID::bigint,'menuGroup_RefID', '254000000000006'::bigint,'menu_RefID', '97000000000067'::bigint)))::varchar;</v>
       </c>
     </row>
     <row r="69" spans="2:11" x14ac:dyDescent="0.2">
@@ -3901,7 +3901,7 @@
       </c>
       <c r="K69" s="2" t="str">
         <f t="shared" si="3"/>
-        <v>varSQL := varSQL || (CASE WHEN (varSQL = '') THEN '' ELSE ', ' END) || (SELECT JSON_BUILD_OBJECT ('recordID', NULL::bigint,'entities', JSON_BUILD_OBJECT ('sysLoginSession_RefID', varSystemLoginSession::bigint,'sysDataAnnotation', NULL::varchar,'sysDataSetDateTimeTZ', NULL::timestamptz,'sysDataValidityStartDateTimeTZ', NULL::timestamptz,'sysDataValidityFinishDateTimeTZ', NULL::timestamptz,'sysPartitionRemovableRecordKey_RefID', NULL::bigint,'sysBranch_RefID', varInstitutionBranchID::bigint,'sysBaseCurrency_RefID',varBaseCurrencyID::bigint,'name', '254000000000006'::varchar,'iconSource', '97000000000068'::varchar)))::varchar;</v>
+        <v>varSQL := varSQL || (CASE WHEN (varSQL = '') THEN '' ELSE ', ' END) || (SELECT JSON_BUILD_OBJECT ('recordID', NULL::bigint,'entities', JSON_BUILD_OBJECT ('sysLoginSession_RefID', varSystemLoginSession::bigint,'sysDataAnnotation', NULL::varchar,'sysDataSetDateTimeTZ', NULL::timestamptz,'sysDataValidityStartDateTimeTZ', NULL::timestamptz,'sysDataValidityFinishDateTimeTZ', NULL::timestamptz,'sysPartitionRemovableRecordKey_RefID', NULL::bigint,'sysBranch_RefID', varInstitutionBranchID::bigint,'sysBaseCurrency_RefID',varBaseCurrencyID::bigint,'menuGroup_RefID', '254000000000006'::bigint,'menu_RefID', '97000000000068'::bigint)))::varchar;</v>
       </c>
     </row>
     <row r="70" spans="2:11" x14ac:dyDescent="0.2">
@@ -3933,7 +3933,7 @@
       </c>
       <c r="K70" s="2" t="str">
         <f t="shared" si="3"/>
-        <v>varSQL := varSQL || (CASE WHEN (varSQL = '') THEN '' ELSE ', ' END) || (SELECT JSON_BUILD_OBJECT ('recordID', NULL::bigint,'entities', JSON_BUILD_OBJECT ('sysLoginSession_RefID', varSystemLoginSession::bigint,'sysDataAnnotation', NULL::varchar,'sysDataSetDateTimeTZ', NULL::timestamptz,'sysDataValidityStartDateTimeTZ', NULL::timestamptz,'sysDataValidityFinishDateTimeTZ', NULL::timestamptz,'sysPartitionRemovableRecordKey_RefID', NULL::bigint,'sysBranch_RefID', varInstitutionBranchID::bigint,'sysBaseCurrency_RefID',varBaseCurrencyID::bigint,'name', '254000000000006'::varchar,'iconSource', '97000000000069'::varchar)))::varchar;</v>
+        <v>varSQL := varSQL || (CASE WHEN (varSQL = '') THEN '' ELSE ', ' END) || (SELECT JSON_BUILD_OBJECT ('recordID', NULL::bigint,'entities', JSON_BUILD_OBJECT ('sysLoginSession_RefID', varSystemLoginSession::bigint,'sysDataAnnotation', NULL::varchar,'sysDataSetDateTimeTZ', NULL::timestamptz,'sysDataValidityStartDateTimeTZ', NULL::timestamptz,'sysDataValidityFinishDateTimeTZ', NULL::timestamptz,'sysPartitionRemovableRecordKey_RefID', NULL::bigint,'sysBranch_RefID', varInstitutionBranchID::bigint,'sysBaseCurrency_RefID',varBaseCurrencyID::bigint,'menuGroup_RefID', '254000000000006'::bigint,'menu_RefID', '97000000000069'::bigint)))::varchar;</v>
       </c>
     </row>
     <row r="71" spans="2:11" x14ac:dyDescent="0.2">
@@ -3965,7 +3965,7 @@
       </c>
       <c r="K71" s="2" t="str">
         <f t="shared" si="3"/>
-        <v>varSQL := varSQL || (CASE WHEN (varSQL = '') THEN '' ELSE ', ' END) || (SELECT JSON_BUILD_OBJECT ('recordID', NULL::bigint,'entities', JSON_BUILD_OBJECT ('sysLoginSession_RefID', varSystemLoginSession::bigint,'sysDataAnnotation', NULL::varchar,'sysDataSetDateTimeTZ', NULL::timestamptz,'sysDataValidityStartDateTimeTZ', NULL::timestamptz,'sysDataValidityFinishDateTimeTZ', NULL::timestamptz,'sysPartitionRemovableRecordKey_RefID', NULL::bigint,'sysBranch_RefID', varInstitutionBranchID::bigint,'sysBaseCurrency_RefID',varBaseCurrencyID::bigint,'name', '254000000000006'::varchar,'iconSource', '97000000000070'::varchar)))::varchar;</v>
+        <v>varSQL := varSQL || (CASE WHEN (varSQL = '') THEN '' ELSE ', ' END) || (SELECT JSON_BUILD_OBJECT ('recordID', NULL::bigint,'entities', JSON_BUILD_OBJECT ('sysLoginSession_RefID', varSystemLoginSession::bigint,'sysDataAnnotation', NULL::varchar,'sysDataSetDateTimeTZ', NULL::timestamptz,'sysDataValidityStartDateTimeTZ', NULL::timestamptz,'sysDataValidityFinishDateTimeTZ', NULL::timestamptz,'sysPartitionRemovableRecordKey_RefID', NULL::bigint,'sysBranch_RefID', varInstitutionBranchID::bigint,'sysBaseCurrency_RefID',varBaseCurrencyID::bigint,'menuGroup_RefID', '254000000000006'::bigint,'menu_RefID', '97000000000070'::bigint)))::varchar;</v>
       </c>
     </row>
     <row r="72" spans="2:11" x14ac:dyDescent="0.2">
@@ -3997,7 +3997,7 @@
       </c>
       <c r="K72" s="2" t="str">
         <f t="shared" si="3"/>
-        <v>varSQL := varSQL || (CASE WHEN (varSQL = '') THEN '' ELSE ', ' END) || (SELECT JSON_BUILD_OBJECT ('recordID', NULL::bigint,'entities', JSON_BUILD_OBJECT ('sysLoginSession_RefID', varSystemLoginSession::bigint,'sysDataAnnotation', NULL::varchar,'sysDataSetDateTimeTZ', NULL::timestamptz,'sysDataValidityStartDateTimeTZ', NULL::timestamptz,'sysDataValidityFinishDateTimeTZ', NULL::timestamptz,'sysPartitionRemovableRecordKey_RefID', NULL::bigint,'sysBranch_RefID', varInstitutionBranchID::bigint,'sysBaseCurrency_RefID',varBaseCurrencyID::bigint,'name', '254000000000006'::varchar,'iconSource', '97000000000071'::varchar)))::varchar;</v>
+        <v>varSQL := varSQL || (CASE WHEN (varSQL = '') THEN '' ELSE ', ' END) || (SELECT JSON_BUILD_OBJECT ('recordID', NULL::bigint,'entities', JSON_BUILD_OBJECT ('sysLoginSession_RefID', varSystemLoginSession::bigint,'sysDataAnnotation', NULL::varchar,'sysDataSetDateTimeTZ', NULL::timestamptz,'sysDataValidityStartDateTimeTZ', NULL::timestamptz,'sysDataValidityFinishDateTimeTZ', NULL::timestamptz,'sysPartitionRemovableRecordKey_RefID', NULL::bigint,'sysBranch_RefID', varInstitutionBranchID::bigint,'sysBaseCurrency_RefID',varBaseCurrencyID::bigint,'menuGroup_RefID', '254000000000006'::bigint,'menu_RefID', '97000000000071'::bigint)))::varchar;</v>
       </c>
     </row>
     <row r="73" spans="2:11" x14ac:dyDescent="0.2">
@@ -4029,7 +4029,7 @@
       </c>
       <c r="K73" s="2" t="str">
         <f t="shared" si="3"/>
-        <v>varSQL := varSQL || (CASE WHEN (varSQL = '') THEN '' ELSE ', ' END) || (SELECT JSON_BUILD_OBJECT ('recordID', NULL::bigint,'entities', JSON_BUILD_OBJECT ('sysLoginSession_RefID', varSystemLoginSession::bigint,'sysDataAnnotation', NULL::varchar,'sysDataSetDateTimeTZ', NULL::timestamptz,'sysDataValidityStartDateTimeTZ', NULL::timestamptz,'sysDataValidityFinishDateTimeTZ', NULL::timestamptz,'sysPartitionRemovableRecordKey_RefID', NULL::bigint,'sysBranch_RefID', varInstitutionBranchID::bigint,'sysBaseCurrency_RefID',varBaseCurrencyID::bigint,'name', '254000000000006'::varchar,'iconSource', '97000000000072'::varchar)))::varchar;</v>
+        <v>varSQL := varSQL || (CASE WHEN (varSQL = '') THEN '' ELSE ', ' END) || (SELECT JSON_BUILD_OBJECT ('recordID', NULL::bigint,'entities', JSON_BUILD_OBJECT ('sysLoginSession_RefID', varSystemLoginSession::bigint,'sysDataAnnotation', NULL::varchar,'sysDataSetDateTimeTZ', NULL::timestamptz,'sysDataValidityStartDateTimeTZ', NULL::timestamptz,'sysDataValidityFinishDateTimeTZ', NULL::timestamptz,'sysPartitionRemovableRecordKey_RefID', NULL::bigint,'sysBranch_RefID', varInstitutionBranchID::bigint,'sysBaseCurrency_RefID',varBaseCurrencyID::bigint,'menuGroup_RefID', '254000000000006'::bigint,'menu_RefID', '97000000000072'::bigint)))::varchar;</v>
       </c>
     </row>
     <row r="74" spans="2:11" x14ac:dyDescent="0.2">
@@ -4061,7 +4061,7 @@
       </c>
       <c r="K74" s="2" t="str">
         <f t="shared" si="3"/>
-        <v>varSQL := varSQL || (CASE WHEN (varSQL = '') THEN '' ELSE ', ' END) || (SELECT JSON_BUILD_OBJECT ('recordID', NULL::bigint,'entities', JSON_BUILD_OBJECT ('sysLoginSession_RefID', varSystemLoginSession::bigint,'sysDataAnnotation', NULL::varchar,'sysDataSetDateTimeTZ', NULL::timestamptz,'sysDataValidityStartDateTimeTZ', NULL::timestamptz,'sysDataValidityFinishDateTimeTZ', NULL::timestamptz,'sysPartitionRemovableRecordKey_RefID', NULL::bigint,'sysBranch_RefID', varInstitutionBranchID::bigint,'sysBaseCurrency_RefID',varBaseCurrencyID::bigint,'name', '254000000000006'::varchar,'iconSource', '97000000000073'::varchar)))::varchar;</v>
+        <v>varSQL := varSQL || (CASE WHEN (varSQL = '') THEN '' ELSE ', ' END) || (SELECT JSON_BUILD_OBJECT ('recordID', NULL::bigint,'entities', JSON_BUILD_OBJECT ('sysLoginSession_RefID', varSystemLoginSession::bigint,'sysDataAnnotation', NULL::varchar,'sysDataSetDateTimeTZ', NULL::timestamptz,'sysDataValidityStartDateTimeTZ', NULL::timestamptz,'sysDataValidityFinishDateTimeTZ', NULL::timestamptz,'sysPartitionRemovableRecordKey_RefID', NULL::bigint,'sysBranch_RefID', varInstitutionBranchID::bigint,'sysBaseCurrency_RefID',varBaseCurrencyID::bigint,'menuGroup_RefID', '254000000000006'::bigint,'menu_RefID', '97000000000073'::bigint)))::varchar;</v>
       </c>
     </row>
     <row r="75" spans="2:11" x14ac:dyDescent="0.2">
@@ -4093,7 +4093,7 @@
       </c>
       <c r="K75" s="2" t="str">
         <f t="shared" si="3"/>
-        <v>varSQL := varSQL || (CASE WHEN (varSQL = '') THEN '' ELSE ', ' END) || (SELECT JSON_BUILD_OBJECT ('recordID', NULL::bigint,'entities', JSON_BUILD_OBJECT ('sysLoginSession_RefID', varSystemLoginSession::bigint,'sysDataAnnotation', NULL::varchar,'sysDataSetDateTimeTZ', NULL::timestamptz,'sysDataValidityStartDateTimeTZ', NULL::timestamptz,'sysDataValidityFinishDateTimeTZ', NULL::timestamptz,'sysPartitionRemovableRecordKey_RefID', NULL::bigint,'sysBranch_RefID', varInstitutionBranchID::bigint,'sysBaseCurrency_RefID',varBaseCurrencyID::bigint,'name', '254000000000006'::varchar,'iconSource', '97000000000074'::varchar)))::varchar;</v>
+        <v>varSQL := varSQL || (CASE WHEN (varSQL = '') THEN '' ELSE ', ' END) || (SELECT JSON_BUILD_OBJECT ('recordID', NULL::bigint,'entities', JSON_BUILD_OBJECT ('sysLoginSession_RefID', varSystemLoginSession::bigint,'sysDataAnnotation', NULL::varchar,'sysDataSetDateTimeTZ', NULL::timestamptz,'sysDataValidityStartDateTimeTZ', NULL::timestamptz,'sysDataValidityFinishDateTimeTZ', NULL::timestamptz,'sysPartitionRemovableRecordKey_RefID', NULL::bigint,'sysBranch_RefID', varInstitutionBranchID::bigint,'sysBaseCurrency_RefID',varBaseCurrencyID::bigint,'menuGroup_RefID', '254000000000006'::bigint,'menu_RefID', '97000000000074'::bigint)))::varchar;</v>
       </c>
     </row>
     <row r="76" spans="2:11" x14ac:dyDescent="0.2">
@@ -4125,7 +4125,7 @@
       </c>
       <c r="K76" s="2" t="str">
         <f t="shared" si="3"/>
-        <v>varSQL := varSQL || (CASE WHEN (varSQL = '') THEN '' ELSE ', ' END) || (SELECT JSON_BUILD_OBJECT ('recordID', NULL::bigint,'entities', JSON_BUILD_OBJECT ('sysLoginSession_RefID', varSystemLoginSession::bigint,'sysDataAnnotation', NULL::varchar,'sysDataSetDateTimeTZ', NULL::timestamptz,'sysDataValidityStartDateTimeTZ', NULL::timestamptz,'sysDataValidityFinishDateTimeTZ', NULL::timestamptz,'sysPartitionRemovableRecordKey_RefID', NULL::bigint,'sysBranch_RefID', varInstitutionBranchID::bigint,'sysBaseCurrency_RefID',varBaseCurrencyID::bigint,'name', '254000000000006'::varchar,'iconSource', '97000000000075'::varchar)))::varchar;</v>
+        <v>varSQL := varSQL || (CASE WHEN (varSQL = '') THEN '' ELSE ', ' END) || (SELECT JSON_BUILD_OBJECT ('recordID', NULL::bigint,'entities', JSON_BUILD_OBJECT ('sysLoginSession_RefID', varSystemLoginSession::bigint,'sysDataAnnotation', NULL::varchar,'sysDataSetDateTimeTZ', NULL::timestamptz,'sysDataValidityStartDateTimeTZ', NULL::timestamptz,'sysDataValidityFinishDateTimeTZ', NULL::timestamptz,'sysPartitionRemovableRecordKey_RefID', NULL::bigint,'sysBranch_RefID', varInstitutionBranchID::bigint,'sysBaseCurrency_RefID',varBaseCurrencyID::bigint,'menuGroup_RefID', '254000000000006'::bigint,'menu_RefID', '97000000000075'::bigint)))::varchar;</v>
       </c>
     </row>
     <row r="77" spans="2:11" x14ac:dyDescent="0.2">
@@ -4157,7 +4157,7 @@
       </c>
       <c r="K77" s="2" t="str">
         <f t="shared" si="3"/>
-        <v>varSQL := varSQL || (CASE WHEN (varSQL = '') THEN '' ELSE ', ' END) || (SELECT JSON_BUILD_OBJECT ('recordID', NULL::bigint,'entities', JSON_BUILD_OBJECT ('sysLoginSession_RefID', varSystemLoginSession::bigint,'sysDataAnnotation', NULL::varchar,'sysDataSetDateTimeTZ', NULL::timestamptz,'sysDataValidityStartDateTimeTZ', NULL::timestamptz,'sysDataValidityFinishDateTimeTZ', NULL::timestamptz,'sysPartitionRemovableRecordKey_RefID', NULL::bigint,'sysBranch_RefID', varInstitutionBranchID::bigint,'sysBaseCurrency_RefID',varBaseCurrencyID::bigint,'name', '254000000000006'::varchar,'iconSource', '97000000000076'::varchar)))::varchar;</v>
+        <v>varSQL := varSQL || (CASE WHEN (varSQL = '') THEN '' ELSE ', ' END) || (SELECT JSON_BUILD_OBJECT ('recordID', NULL::bigint,'entities', JSON_BUILD_OBJECT ('sysLoginSession_RefID', varSystemLoginSession::bigint,'sysDataAnnotation', NULL::varchar,'sysDataSetDateTimeTZ', NULL::timestamptz,'sysDataValidityStartDateTimeTZ', NULL::timestamptz,'sysDataValidityFinishDateTimeTZ', NULL::timestamptz,'sysPartitionRemovableRecordKey_RefID', NULL::bigint,'sysBranch_RefID', varInstitutionBranchID::bigint,'sysBaseCurrency_RefID',varBaseCurrencyID::bigint,'menuGroup_RefID', '254000000000006'::bigint,'menu_RefID', '97000000000076'::bigint)))::varchar;</v>
       </c>
     </row>
     <row r="78" spans="2:11" x14ac:dyDescent="0.2">
@@ -4189,7 +4189,7 @@
       </c>
       <c r="K78" s="2" t="str">
         <f t="shared" si="3"/>
-        <v>varSQL := varSQL || (CASE WHEN (varSQL = '') THEN '' ELSE ', ' END) || (SELECT JSON_BUILD_OBJECT ('recordID', NULL::bigint,'entities', JSON_BUILD_OBJECT ('sysLoginSession_RefID', varSystemLoginSession::bigint,'sysDataAnnotation', NULL::varchar,'sysDataSetDateTimeTZ', NULL::timestamptz,'sysDataValidityStartDateTimeTZ', NULL::timestamptz,'sysDataValidityFinishDateTimeTZ', NULL::timestamptz,'sysPartitionRemovableRecordKey_RefID', NULL::bigint,'sysBranch_RefID', varInstitutionBranchID::bigint,'sysBaseCurrency_RefID',varBaseCurrencyID::bigint,'name', '254000000000006'::varchar,'iconSource', '97000000000077'::varchar)))::varchar;</v>
+        <v>varSQL := varSQL || (CASE WHEN (varSQL = '') THEN '' ELSE ', ' END) || (SELECT JSON_BUILD_OBJECT ('recordID', NULL::bigint,'entities', JSON_BUILD_OBJECT ('sysLoginSession_RefID', varSystemLoginSession::bigint,'sysDataAnnotation', NULL::varchar,'sysDataSetDateTimeTZ', NULL::timestamptz,'sysDataValidityStartDateTimeTZ', NULL::timestamptz,'sysDataValidityFinishDateTimeTZ', NULL::timestamptz,'sysPartitionRemovableRecordKey_RefID', NULL::bigint,'sysBranch_RefID', varInstitutionBranchID::bigint,'sysBaseCurrency_RefID',varBaseCurrencyID::bigint,'menuGroup_RefID', '254000000000006'::bigint,'menu_RefID', '97000000000077'::bigint)))::varchar;</v>
       </c>
     </row>
     <row r="79" spans="2:11" x14ac:dyDescent="0.2">
@@ -4221,7 +4221,7 @@
       </c>
       <c r="K79" s="2" t="str">
         <f t="shared" si="3"/>
-        <v>varSQL := varSQL || (CASE WHEN (varSQL = '') THEN '' ELSE ', ' END) || (SELECT JSON_BUILD_OBJECT ('recordID', NULL::bigint,'entities', JSON_BUILD_OBJECT ('sysLoginSession_RefID', varSystemLoginSession::bigint,'sysDataAnnotation', NULL::varchar,'sysDataSetDateTimeTZ', NULL::timestamptz,'sysDataValidityStartDateTimeTZ', NULL::timestamptz,'sysDataValidityFinishDateTimeTZ', NULL::timestamptz,'sysPartitionRemovableRecordKey_RefID', NULL::bigint,'sysBranch_RefID', varInstitutionBranchID::bigint,'sysBaseCurrency_RefID',varBaseCurrencyID::bigint,'name', '254000000000006'::varchar,'iconSource', '97000000000078'::varchar)))::varchar;</v>
+        <v>varSQL := varSQL || (CASE WHEN (varSQL = '') THEN '' ELSE ', ' END) || (SELECT JSON_BUILD_OBJECT ('recordID', NULL::bigint,'entities', JSON_BUILD_OBJECT ('sysLoginSession_RefID', varSystemLoginSession::bigint,'sysDataAnnotation', NULL::varchar,'sysDataSetDateTimeTZ', NULL::timestamptz,'sysDataValidityStartDateTimeTZ', NULL::timestamptz,'sysDataValidityFinishDateTimeTZ', NULL::timestamptz,'sysPartitionRemovableRecordKey_RefID', NULL::bigint,'sysBranch_RefID', varInstitutionBranchID::bigint,'sysBaseCurrency_RefID',varBaseCurrencyID::bigint,'menuGroup_RefID', '254000000000006'::bigint,'menu_RefID', '97000000000078'::bigint)))::varchar;</v>
       </c>
     </row>
     <row r="80" spans="2:11" x14ac:dyDescent="0.2">
@@ -4253,7 +4253,7 @@
       </c>
       <c r="K80" s="2" t="str">
         <f t="shared" si="3"/>
-        <v>varSQL := varSQL || (CASE WHEN (varSQL = '') THEN '' ELSE ', ' END) || (SELECT JSON_BUILD_OBJECT ('recordID', NULL::bigint,'entities', JSON_BUILD_OBJECT ('sysLoginSession_RefID', varSystemLoginSession::bigint,'sysDataAnnotation', NULL::varchar,'sysDataSetDateTimeTZ', NULL::timestamptz,'sysDataValidityStartDateTimeTZ', NULL::timestamptz,'sysDataValidityFinishDateTimeTZ', NULL::timestamptz,'sysPartitionRemovableRecordKey_RefID', NULL::bigint,'sysBranch_RefID', varInstitutionBranchID::bigint,'sysBaseCurrency_RefID',varBaseCurrencyID::bigint,'name', '254000000000006'::varchar,'iconSource', '97000000000079'::varchar)))::varchar;</v>
+        <v>varSQL := varSQL || (CASE WHEN (varSQL = '') THEN '' ELSE ', ' END) || (SELECT JSON_BUILD_OBJECT ('recordID', NULL::bigint,'entities', JSON_BUILD_OBJECT ('sysLoginSession_RefID', varSystemLoginSession::bigint,'sysDataAnnotation', NULL::varchar,'sysDataSetDateTimeTZ', NULL::timestamptz,'sysDataValidityStartDateTimeTZ', NULL::timestamptz,'sysDataValidityFinishDateTimeTZ', NULL::timestamptz,'sysPartitionRemovableRecordKey_RefID', NULL::bigint,'sysBranch_RefID', varInstitutionBranchID::bigint,'sysBaseCurrency_RefID',varBaseCurrencyID::bigint,'menuGroup_RefID', '254000000000006'::bigint,'menu_RefID', '97000000000079'::bigint)))::varchar;</v>
       </c>
     </row>
     <row r="81" spans="2:11" x14ac:dyDescent="0.2">
@@ -4285,7 +4285,7 @@
       </c>
       <c r="K81" s="2" t="str">
         <f t="shared" si="3"/>
-        <v>varSQL := varSQL || (CASE WHEN (varSQL = '') THEN '' ELSE ', ' END) || (SELECT JSON_BUILD_OBJECT ('recordID', NULL::bigint,'entities', JSON_BUILD_OBJECT ('sysLoginSession_RefID', varSystemLoginSession::bigint,'sysDataAnnotation', NULL::varchar,'sysDataSetDateTimeTZ', NULL::timestamptz,'sysDataValidityStartDateTimeTZ', NULL::timestamptz,'sysDataValidityFinishDateTimeTZ', NULL::timestamptz,'sysPartitionRemovableRecordKey_RefID', NULL::bigint,'sysBranch_RefID', varInstitutionBranchID::bigint,'sysBaseCurrency_RefID',varBaseCurrencyID::bigint,'name', '254000000000006'::varchar,'iconSource', '97000000000080'::varchar)))::varchar;</v>
+        <v>varSQL := varSQL || (CASE WHEN (varSQL = '') THEN '' ELSE ', ' END) || (SELECT JSON_BUILD_OBJECT ('recordID', NULL::bigint,'entities', JSON_BUILD_OBJECT ('sysLoginSession_RefID', varSystemLoginSession::bigint,'sysDataAnnotation', NULL::varchar,'sysDataSetDateTimeTZ', NULL::timestamptz,'sysDataValidityStartDateTimeTZ', NULL::timestamptz,'sysDataValidityFinishDateTimeTZ', NULL::timestamptz,'sysPartitionRemovableRecordKey_RefID', NULL::bigint,'sysBranch_RefID', varInstitutionBranchID::bigint,'sysBaseCurrency_RefID',varBaseCurrencyID::bigint,'menuGroup_RefID', '254000000000006'::bigint,'menu_RefID', '97000000000080'::bigint)))::varchar;</v>
       </c>
     </row>
     <row r="82" spans="2:11" x14ac:dyDescent="0.2">
@@ -4317,7 +4317,7 @@
       </c>
       <c r="K82" s="2" t="str">
         <f t="shared" si="3"/>
-        <v>varSQL := varSQL || (CASE WHEN (varSQL = '') THEN '' ELSE ', ' END) || (SELECT JSON_BUILD_OBJECT ('recordID', NULL::bigint,'entities', JSON_BUILD_OBJECT ('sysLoginSession_RefID', varSystemLoginSession::bigint,'sysDataAnnotation', NULL::varchar,'sysDataSetDateTimeTZ', NULL::timestamptz,'sysDataValidityStartDateTimeTZ', NULL::timestamptz,'sysDataValidityFinishDateTimeTZ', NULL::timestamptz,'sysPartitionRemovableRecordKey_RefID', NULL::bigint,'sysBranch_RefID', varInstitutionBranchID::bigint,'sysBaseCurrency_RefID',varBaseCurrencyID::bigint,'name', '254000000000006'::varchar,'iconSource', '97000000000081'::varchar)))::varchar;</v>
+        <v>varSQL := varSQL || (CASE WHEN (varSQL = '') THEN '' ELSE ', ' END) || (SELECT JSON_BUILD_OBJECT ('recordID', NULL::bigint,'entities', JSON_BUILD_OBJECT ('sysLoginSession_RefID', varSystemLoginSession::bigint,'sysDataAnnotation', NULL::varchar,'sysDataSetDateTimeTZ', NULL::timestamptz,'sysDataValidityStartDateTimeTZ', NULL::timestamptz,'sysDataValidityFinishDateTimeTZ', NULL::timestamptz,'sysPartitionRemovableRecordKey_RefID', NULL::bigint,'sysBranch_RefID', varInstitutionBranchID::bigint,'sysBaseCurrency_RefID',varBaseCurrencyID::bigint,'menuGroup_RefID', '254000000000006'::bigint,'menu_RefID', '97000000000081'::bigint)))::varchar;</v>
       </c>
     </row>
     <row r="83" spans="2:11" x14ac:dyDescent="0.2">
@@ -4349,7 +4349,7 @@
       </c>
       <c r="K83" s="2" t="str">
         <f t="shared" si="3"/>
-        <v>varSQL := varSQL || (CASE WHEN (varSQL = '') THEN '' ELSE ', ' END) || (SELECT JSON_BUILD_OBJECT ('recordID', NULL::bigint,'entities', JSON_BUILD_OBJECT ('sysLoginSession_RefID', varSystemLoginSession::bigint,'sysDataAnnotation', NULL::varchar,'sysDataSetDateTimeTZ', NULL::timestamptz,'sysDataValidityStartDateTimeTZ', NULL::timestamptz,'sysDataValidityFinishDateTimeTZ', NULL::timestamptz,'sysPartitionRemovableRecordKey_RefID', NULL::bigint,'sysBranch_RefID', varInstitutionBranchID::bigint,'sysBaseCurrency_RefID',varBaseCurrencyID::bigint,'name', '254000000000006'::varchar,'iconSource', '97000000000082'::varchar)))::varchar;</v>
+        <v>varSQL := varSQL || (CASE WHEN (varSQL = '') THEN '' ELSE ', ' END) || (SELECT JSON_BUILD_OBJECT ('recordID', NULL::bigint,'entities', JSON_BUILD_OBJECT ('sysLoginSession_RefID', varSystemLoginSession::bigint,'sysDataAnnotation', NULL::varchar,'sysDataSetDateTimeTZ', NULL::timestamptz,'sysDataValidityStartDateTimeTZ', NULL::timestamptz,'sysDataValidityFinishDateTimeTZ', NULL::timestamptz,'sysPartitionRemovableRecordKey_RefID', NULL::bigint,'sysBranch_RefID', varInstitutionBranchID::bigint,'sysBaseCurrency_RefID',varBaseCurrencyID::bigint,'menuGroup_RefID', '254000000000006'::bigint,'menu_RefID', '97000000000082'::bigint)))::varchar;</v>
       </c>
     </row>
     <row r="84" spans="2:11" x14ac:dyDescent="0.2">
@@ -4381,7 +4381,7 @@
       </c>
       <c r="K84" s="2" t="str">
         <f t="shared" si="3"/>
-        <v>varSQL := varSQL || (CASE WHEN (varSQL = '') THEN '' ELSE ', ' END) || (SELECT JSON_BUILD_OBJECT ('recordID', NULL::bigint,'entities', JSON_BUILD_OBJECT ('sysLoginSession_RefID', varSystemLoginSession::bigint,'sysDataAnnotation', NULL::varchar,'sysDataSetDateTimeTZ', NULL::timestamptz,'sysDataValidityStartDateTimeTZ', NULL::timestamptz,'sysDataValidityFinishDateTimeTZ', NULL::timestamptz,'sysPartitionRemovableRecordKey_RefID', NULL::bigint,'sysBranch_RefID', varInstitutionBranchID::bigint,'sysBaseCurrency_RefID',varBaseCurrencyID::bigint,'name', '254000000000006'::varchar,'iconSource', '97000000000083'::varchar)))::varchar;</v>
+        <v>varSQL := varSQL || (CASE WHEN (varSQL = '') THEN '' ELSE ', ' END) || (SELECT JSON_BUILD_OBJECT ('recordID', NULL::bigint,'entities', JSON_BUILD_OBJECT ('sysLoginSession_RefID', varSystemLoginSession::bigint,'sysDataAnnotation', NULL::varchar,'sysDataSetDateTimeTZ', NULL::timestamptz,'sysDataValidityStartDateTimeTZ', NULL::timestamptz,'sysDataValidityFinishDateTimeTZ', NULL::timestamptz,'sysPartitionRemovableRecordKey_RefID', NULL::bigint,'sysBranch_RefID', varInstitutionBranchID::bigint,'sysBaseCurrency_RefID',varBaseCurrencyID::bigint,'menuGroup_RefID', '254000000000006'::bigint,'menu_RefID', '97000000000083'::bigint)))::varchar;</v>
       </c>
     </row>
     <row r="85" spans="2:11" x14ac:dyDescent="0.2">
@@ -4413,7 +4413,7 @@
       </c>
       <c r="K85" s="2" t="str">
         <f t="shared" si="3"/>
-        <v>varSQL := varSQL || (CASE WHEN (varSQL = '') THEN '' ELSE ', ' END) || (SELECT JSON_BUILD_OBJECT ('recordID', NULL::bigint,'entities', JSON_BUILD_OBJECT ('sysLoginSession_RefID', varSystemLoginSession::bigint,'sysDataAnnotation', NULL::varchar,'sysDataSetDateTimeTZ', NULL::timestamptz,'sysDataValidityStartDateTimeTZ', NULL::timestamptz,'sysDataValidityFinishDateTimeTZ', NULL::timestamptz,'sysPartitionRemovableRecordKey_RefID', NULL::bigint,'sysBranch_RefID', varInstitutionBranchID::bigint,'sysBaseCurrency_RefID',varBaseCurrencyID::bigint,'name', '254000000000006'::varchar,'iconSource', '97000000000084'::varchar)))::varchar;</v>
+        <v>varSQL := varSQL || (CASE WHEN (varSQL = '') THEN '' ELSE ', ' END) || (SELECT JSON_BUILD_OBJECT ('recordID', NULL::bigint,'entities', JSON_BUILD_OBJECT ('sysLoginSession_RefID', varSystemLoginSession::bigint,'sysDataAnnotation', NULL::varchar,'sysDataSetDateTimeTZ', NULL::timestamptz,'sysDataValidityStartDateTimeTZ', NULL::timestamptz,'sysDataValidityFinishDateTimeTZ', NULL::timestamptz,'sysPartitionRemovableRecordKey_RefID', NULL::bigint,'sysBranch_RefID', varInstitutionBranchID::bigint,'sysBaseCurrency_RefID',varBaseCurrencyID::bigint,'menuGroup_RefID', '254000000000006'::bigint,'menu_RefID', '97000000000084'::bigint)))::varchar;</v>
       </c>
     </row>
     <row r="86" spans="2:11" x14ac:dyDescent="0.2">
@@ -4445,7 +4445,7 @@
       </c>
       <c r="K86" s="2" t="str">
         <f t="shared" si="3"/>
-        <v>varSQL := varSQL || (CASE WHEN (varSQL = '') THEN '' ELSE ', ' END) || (SELECT JSON_BUILD_OBJECT ('recordID', NULL::bigint,'entities', JSON_BUILD_OBJECT ('sysLoginSession_RefID', varSystemLoginSession::bigint,'sysDataAnnotation', NULL::varchar,'sysDataSetDateTimeTZ', NULL::timestamptz,'sysDataValidityStartDateTimeTZ', NULL::timestamptz,'sysDataValidityFinishDateTimeTZ', NULL::timestamptz,'sysPartitionRemovableRecordKey_RefID', NULL::bigint,'sysBranch_RefID', varInstitutionBranchID::bigint,'sysBaseCurrency_RefID',varBaseCurrencyID::bigint,'name', '254000000000006'::varchar,'iconSource', '97000000000085'::varchar)))::varchar;</v>
+        <v>varSQL := varSQL || (CASE WHEN (varSQL = '') THEN '' ELSE ', ' END) || (SELECT JSON_BUILD_OBJECT ('recordID', NULL::bigint,'entities', JSON_BUILD_OBJECT ('sysLoginSession_RefID', varSystemLoginSession::bigint,'sysDataAnnotation', NULL::varchar,'sysDataSetDateTimeTZ', NULL::timestamptz,'sysDataValidityStartDateTimeTZ', NULL::timestamptz,'sysDataValidityFinishDateTimeTZ', NULL::timestamptz,'sysPartitionRemovableRecordKey_RefID', NULL::bigint,'sysBranch_RefID', varInstitutionBranchID::bigint,'sysBaseCurrency_RefID',varBaseCurrencyID::bigint,'menuGroup_RefID', '254000000000006'::bigint,'menu_RefID', '97000000000085'::bigint)))::varchar;</v>
       </c>
     </row>
     <row r="87" spans="2:11" x14ac:dyDescent="0.2">
@@ -4477,7 +4477,7 @@
       </c>
       <c r="K87" s="2" t="str">
         <f t="shared" si="3"/>
-        <v>varSQL := varSQL || (CASE WHEN (varSQL = '') THEN '' ELSE ', ' END) || (SELECT JSON_BUILD_OBJECT ('recordID', NULL::bigint,'entities', JSON_BUILD_OBJECT ('sysLoginSession_RefID', varSystemLoginSession::bigint,'sysDataAnnotation', NULL::varchar,'sysDataSetDateTimeTZ', NULL::timestamptz,'sysDataValidityStartDateTimeTZ', NULL::timestamptz,'sysDataValidityFinishDateTimeTZ', NULL::timestamptz,'sysPartitionRemovableRecordKey_RefID', NULL::bigint,'sysBranch_RefID', varInstitutionBranchID::bigint,'sysBaseCurrency_RefID',varBaseCurrencyID::bigint,'name', '254000000000006'::varchar,'iconSource', '97000000000086'::varchar)))::varchar;</v>
+        <v>varSQL := varSQL || (CASE WHEN (varSQL = '') THEN '' ELSE ', ' END) || (SELECT JSON_BUILD_OBJECT ('recordID', NULL::bigint,'entities', JSON_BUILD_OBJECT ('sysLoginSession_RefID', varSystemLoginSession::bigint,'sysDataAnnotation', NULL::varchar,'sysDataSetDateTimeTZ', NULL::timestamptz,'sysDataValidityStartDateTimeTZ', NULL::timestamptz,'sysDataValidityFinishDateTimeTZ', NULL::timestamptz,'sysPartitionRemovableRecordKey_RefID', NULL::bigint,'sysBranch_RefID', varInstitutionBranchID::bigint,'sysBaseCurrency_RefID',varBaseCurrencyID::bigint,'menuGroup_RefID', '254000000000006'::bigint,'menu_RefID', '97000000000086'::bigint)))::varchar;</v>
       </c>
     </row>
     <row r="88" spans="2:11" x14ac:dyDescent="0.2">
@@ -4509,7 +4509,7 @@
       </c>
       <c r="K88" s="2" t="str">
         <f t="shared" si="3"/>
-        <v>varSQL := varSQL || (CASE WHEN (varSQL = '') THEN '' ELSE ', ' END) || (SELECT JSON_BUILD_OBJECT ('recordID', NULL::bigint,'entities', JSON_BUILD_OBJECT ('sysLoginSession_RefID', varSystemLoginSession::bigint,'sysDataAnnotation', NULL::varchar,'sysDataSetDateTimeTZ', NULL::timestamptz,'sysDataValidityStartDateTimeTZ', NULL::timestamptz,'sysDataValidityFinishDateTimeTZ', NULL::timestamptz,'sysPartitionRemovableRecordKey_RefID', NULL::bigint,'sysBranch_RefID', varInstitutionBranchID::bigint,'sysBaseCurrency_RefID',varBaseCurrencyID::bigint,'name', '254000000000006'::varchar,'iconSource', '97000000000087'::varchar)))::varchar;</v>
+        <v>varSQL := varSQL || (CASE WHEN (varSQL = '') THEN '' ELSE ', ' END) || (SELECT JSON_BUILD_OBJECT ('recordID', NULL::bigint,'entities', JSON_BUILD_OBJECT ('sysLoginSession_RefID', varSystemLoginSession::bigint,'sysDataAnnotation', NULL::varchar,'sysDataSetDateTimeTZ', NULL::timestamptz,'sysDataValidityStartDateTimeTZ', NULL::timestamptz,'sysDataValidityFinishDateTimeTZ', NULL::timestamptz,'sysPartitionRemovableRecordKey_RefID', NULL::bigint,'sysBranch_RefID', varInstitutionBranchID::bigint,'sysBaseCurrency_RefID',varBaseCurrencyID::bigint,'menuGroup_RefID', '254000000000006'::bigint,'menu_RefID', '97000000000087'::bigint)))::varchar;</v>
       </c>
     </row>
     <row r="89" spans="2:11" x14ac:dyDescent="0.2">
@@ -4541,7 +4541,7 @@
       </c>
       <c r="K89" s="2" t="str">
         <f t="shared" si="3"/>
-        <v>varSQL := varSQL || (CASE WHEN (varSQL = '') THEN '' ELSE ', ' END) || (SELECT JSON_BUILD_OBJECT ('recordID', NULL::bigint,'entities', JSON_BUILD_OBJECT ('sysLoginSession_RefID', varSystemLoginSession::bigint,'sysDataAnnotation', NULL::varchar,'sysDataSetDateTimeTZ', NULL::timestamptz,'sysDataValidityStartDateTimeTZ', NULL::timestamptz,'sysDataValidityFinishDateTimeTZ', NULL::timestamptz,'sysPartitionRemovableRecordKey_RefID', NULL::bigint,'sysBranch_RefID', varInstitutionBranchID::bigint,'sysBaseCurrency_RefID',varBaseCurrencyID::bigint,'name', '254000000000006'::varchar,'iconSource', '97000000000088'::varchar)))::varchar;</v>
+        <v>varSQL := varSQL || (CASE WHEN (varSQL = '') THEN '' ELSE ', ' END) || (SELECT JSON_BUILD_OBJECT ('recordID', NULL::bigint,'entities', JSON_BUILD_OBJECT ('sysLoginSession_RefID', varSystemLoginSession::bigint,'sysDataAnnotation', NULL::varchar,'sysDataSetDateTimeTZ', NULL::timestamptz,'sysDataValidityStartDateTimeTZ', NULL::timestamptz,'sysDataValidityFinishDateTimeTZ', NULL::timestamptz,'sysPartitionRemovableRecordKey_RefID', NULL::bigint,'sysBranch_RefID', varInstitutionBranchID::bigint,'sysBaseCurrency_RefID',varBaseCurrencyID::bigint,'menuGroup_RefID', '254000000000006'::bigint,'menu_RefID', '97000000000088'::bigint)))::varchar;</v>
       </c>
     </row>
     <row r="90" spans="2:11" x14ac:dyDescent="0.2">
@@ -4573,7 +4573,7 @@
       </c>
       <c r="K90" s="2" t="str">
         <f t="shared" si="3"/>
-        <v>varSQL := varSQL || (CASE WHEN (varSQL = '') THEN '' ELSE ', ' END) || (SELECT JSON_BUILD_OBJECT ('recordID', NULL::bigint,'entities', JSON_BUILD_OBJECT ('sysLoginSession_RefID', varSystemLoginSession::bigint,'sysDataAnnotation', NULL::varchar,'sysDataSetDateTimeTZ', NULL::timestamptz,'sysDataValidityStartDateTimeTZ', NULL::timestamptz,'sysDataValidityFinishDateTimeTZ', NULL::timestamptz,'sysPartitionRemovableRecordKey_RefID', NULL::bigint,'sysBranch_RefID', varInstitutionBranchID::bigint,'sysBaseCurrency_RefID',varBaseCurrencyID::bigint,'name', '254000000000006'::varchar,'iconSource', '97000000000089'::varchar)))::varchar;</v>
+        <v>varSQL := varSQL || (CASE WHEN (varSQL = '') THEN '' ELSE ', ' END) || (SELECT JSON_BUILD_OBJECT ('recordID', NULL::bigint,'entities', JSON_BUILD_OBJECT ('sysLoginSession_RefID', varSystemLoginSession::bigint,'sysDataAnnotation', NULL::varchar,'sysDataSetDateTimeTZ', NULL::timestamptz,'sysDataValidityStartDateTimeTZ', NULL::timestamptz,'sysDataValidityFinishDateTimeTZ', NULL::timestamptz,'sysPartitionRemovableRecordKey_RefID', NULL::bigint,'sysBranch_RefID', varInstitutionBranchID::bigint,'sysBaseCurrency_RefID',varBaseCurrencyID::bigint,'menuGroup_RefID', '254000000000006'::bigint,'menu_RefID', '97000000000089'::bigint)))::varchar;</v>
       </c>
     </row>
     <row r="91" spans="2:11" x14ac:dyDescent="0.2">
@@ -4605,7 +4605,7 @@
       </c>
       <c r="K91" s="2" t="str">
         <f t="shared" si="3"/>
-        <v>varSQL := varSQL || (CASE WHEN (varSQL = '') THEN '' ELSE ', ' END) || (SELECT JSON_BUILD_OBJECT ('recordID', NULL::bigint,'entities', JSON_BUILD_OBJECT ('sysLoginSession_RefID', varSystemLoginSession::bigint,'sysDataAnnotation', NULL::varchar,'sysDataSetDateTimeTZ', NULL::timestamptz,'sysDataValidityStartDateTimeTZ', NULL::timestamptz,'sysDataValidityFinishDateTimeTZ', NULL::timestamptz,'sysPartitionRemovableRecordKey_RefID', NULL::bigint,'sysBranch_RefID', varInstitutionBranchID::bigint,'sysBaseCurrency_RefID',varBaseCurrencyID::bigint,'name', '254000000000006'::varchar,'iconSource', '97000000000090'::varchar)))::varchar;</v>
+        <v>varSQL := varSQL || (CASE WHEN (varSQL = '') THEN '' ELSE ', ' END) || (SELECT JSON_BUILD_OBJECT ('recordID', NULL::bigint,'entities', JSON_BUILD_OBJECT ('sysLoginSession_RefID', varSystemLoginSession::bigint,'sysDataAnnotation', NULL::varchar,'sysDataSetDateTimeTZ', NULL::timestamptz,'sysDataValidityStartDateTimeTZ', NULL::timestamptz,'sysDataValidityFinishDateTimeTZ', NULL::timestamptz,'sysPartitionRemovableRecordKey_RefID', NULL::bigint,'sysBranch_RefID', varInstitutionBranchID::bigint,'sysBaseCurrency_RefID',varBaseCurrencyID::bigint,'menuGroup_RefID', '254000000000006'::bigint,'menu_RefID', '97000000000090'::bigint)))::varchar;</v>
       </c>
     </row>
     <row r="92" spans="2:11" x14ac:dyDescent="0.2">
@@ -4637,7 +4637,7 @@
       </c>
       <c r="K92" s="2" t="str">
         <f t="shared" si="3"/>
-        <v>varSQL := varSQL || (CASE WHEN (varSQL = '') THEN '' ELSE ', ' END) || (SELECT JSON_BUILD_OBJECT ('recordID', NULL::bigint,'entities', JSON_BUILD_OBJECT ('sysLoginSession_RefID', varSystemLoginSession::bigint,'sysDataAnnotation', NULL::varchar,'sysDataSetDateTimeTZ', NULL::timestamptz,'sysDataValidityStartDateTimeTZ', NULL::timestamptz,'sysDataValidityFinishDateTimeTZ', NULL::timestamptz,'sysPartitionRemovableRecordKey_RefID', NULL::bigint,'sysBranch_RefID', varInstitutionBranchID::bigint,'sysBaseCurrency_RefID',varBaseCurrencyID::bigint,'name', '254000000000006'::varchar,'iconSource', '97000000000091'::varchar)))::varchar;</v>
+        <v>varSQL := varSQL || (CASE WHEN (varSQL = '') THEN '' ELSE ', ' END) || (SELECT JSON_BUILD_OBJECT ('recordID', NULL::bigint,'entities', JSON_BUILD_OBJECT ('sysLoginSession_RefID', varSystemLoginSession::bigint,'sysDataAnnotation', NULL::varchar,'sysDataSetDateTimeTZ', NULL::timestamptz,'sysDataValidityStartDateTimeTZ', NULL::timestamptz,'sysDataValidityFinishDateTimeTZ', NULL::timestamptz,'sysPartitionRemovableRecordKey_RefID', NULL::bigint,'sysBranch_RefID', varInstitutionBranchID::bigint,'sysBaseCurrency_RefID',varBaseCurrencyID::bigint,'menuGroup_RefID', '254000000000006'::bigint,'menu_RefID', '97000000000091'::bigint)))::varchar;</v>
       </c>
     </row>
     <row r="93" spans="2:11" x14ac:dyDescent="0.2">
@@ -4669,7 +4669,7 @@
       </c>
       <c r="K93" s="2" t="str">
         <f t="shared" si="3"/>
-        <v>varSQL := varSQL || (CASE WHEN (varSQL = '') THEN '' ELSE ', ' END) || (SELECT JSON_BUILD_OBJECT ('recordID', NULL::bigint,'entities', JSON_BUILD_OBJECT ('sysLoginSession_RefID', varSystemLoginSession::bigint,'sysDataAnnotation', NULL::varchar,'sysDataSetDateTimeTZ', NULL::timestamptz,'sysDataValidityStartDateTimeTZ', NULL::timestamptz,'sysDataValidityFinishDateTimeTZ', NULL::timestamptz,'sysPartitionRemovableRecordKey_RefID', NULL::bigint,'sysBranch_RefID', varInstitutionBranchID::bigint,'sysBaseCurrency_RefID',varBaseCurrencyID::bigint,'name', '254000000000006'::varchar,'iconSource', '97000000000092'::varchar)))::varchar;</v>
+        <v>varSQL := varSQL || (CASE WHEN (varSQL = '') THEN '' ELSE ', ' END) || (SELECT JSON_BUILD_OBJECT ('recordID', NULL::bigint,'entities', JSON_BUILD_OBJECT ('sysLoginSession_RefID', varSystemLoginSession::bigint,'sysDataAnnotation', NULL::varchar,'sysDataSetDateTimeTZ', NULL::timestamptz,'sysDataValidityStartDateTimeTZ', NULL::timestamptz,'sysDataValidityFinishDateTimeTZ', NULL::timestamptz,'sysPartitionRemovableRecordKey_RefID', NULL::bigint,'sysBranch_RefID', varInstitutionBranchID::bigint,'sysBaseCurrency_RefID',varBaseCurrencyID::bigint,'menuGroup_RefID', '254000000000006'::bigint,'menu_RefID', '97000000000092'::bigint)))::varchar;</v>
       </c>
     </row>
     <row r="94" spans="2:11" x14ac:dyDescent="0.2">
@@ -4701,7 +4701,7 @@
       </c>
       <c r="K94" s="2" t="str">
         <f t="shared" si="3"/>
-        <v>varSQL := varSQL || (CASE WHEN (varSQL = '') THEN '' ELSE ', ' END) || (SELECT JSON_BUILD_OBJECT ('recordID', NULL::bigint,'entities', JSON_BUILD_OBJECT ('sysLoginSession_RefID', varSystemLoginSession::bigint,'sysDataAnnotation', NULL::varchar,'sysDataSetDateTimeTZ', NULL::timestamptz,'sysDataValidityStartDateTimeTZ', NULL::timestamptz,'sysDataValidityFinishDateTimeTZ', NULL::timestamptz,'sysPartitionRemovableRecordKey_RefID', NULL::bigint,'sysBranch_RefID', varInstitutionBranchID::bigint,'sysBaseCurrency_RefID',varBaseCurrencyID::bigint,'name', '254000000000006'::varchar,'iconSource', '97000000000093'::varchar)))::varchar;</v>
+        <v>varSQL := varSQL || (CASE WHEN (varSQL = '') THEN '' ELSE ', ' END) || (SELECT JSON_BUILD_OBJECT ('recordID', NULL::bigint,'entities', JSON_BUILD_OBJECT ('sysLoginSession_RefID', varSystemLoginSession::bigint,'sysDataAnnotation', NULL::varchar,'sysDataSetDateTimeTZ', NULL::timestamptz,'sysDataValidityStartDateTimeTZ', NULL::timestamptz,'sysDataValidityFinishDateTimeTZ', NULL::timestamptz,'sysPartitionRemovableRecordKey_RefID', NULL::bigint,'sysBranch_RefID', varInstitutionBranchID::bigint,'sysBaseCurrency_RefID',varBaseCurrencyID::bigint,'menuGroup_RefID', '254000000000006'::bigint,'menu_RefID', '97000000000093'::bigint)))::varchar;</v>
       </c>
     </row>
     <row r="95" spans="2:11" x14ac:dyDescent="0.2">
@@ -4733,7 +4733,7 @@
       </c>
       <c r="K95" s="2" t="str">
         <f t="shared" si="3"/>
-        <v>varSQL := varSQL || (CASE WHEN (varSQL = '') THEN '' ELSE ', ' END) || (SELECT JSON_BUILD_OBJECT ('recordID', NULL::bigint,'entities', JSON_BUILD_OBJECT ('sysLoginSession_RefID', varSystemLoginSession::bigint,'sysDataAnnotation', NULL::varchar,'sysDataSetDateTimeTZ', NULL::timestamptz,'sysDataValidityStartDateTimeTZ', NULL::timestamptz,'sysDataValidityFinishDateTimeTZ', NULL::timestamptz,'sysPartitionRemovableRecordKey_RefID', NULL::bigint,'sysBranch_RefID', varInstitutionBranchID::bigint,'sysBaseCurrency_RefID',varBaseCurrencyID::bigint,'name', '254000000000006'::varchar,'iconSource', '97000000000094'::varchar)))::varchar;</v>
+        <v>varSQL := varSQL || (CASE WHEN (varSQL = '') THEN '' ELSE ', ' END) || (SELECT JSON_BUILD_OBJECT ('recordID', NULL::bigint,'entities', JSON_BUILD_OBJECT ('sysLoginSession_RefID', varSystemLoginSession::bigint,'sysDataAnnotation', NULL::varchar,'sysDataSetDateTimeTZ', NULL::timestamptz,'sysDataValidityStartDateTimeTZ', NULL::timestamptz,'sysDataValidityFinishDateTimeTZ', NULL::timestamptz,'sysPartitionRemovableRecordKey_RefID', NULL::bigint,'sysBranch_RefID', varInstitutionBranchID::bigint,'sysBaseCurrency_RefID',varBaseCurrencyID::bigint,'menuGroup_RefID', '254000000000006'::bigint,'menu_RefID', '97000000000094'::bigint)))::varchar;</v>
       </c>
     </row>
     <row r="96" spans="2:11" x14ac:dyDescent="0.2">
@@ -4765,7 +4765,7 @@
       </c>
       <c r="K96" s="2" t="str">
         <f t="shared" si="3"/>
-        <v>varSQL := varSQL || (CASE WHEN (varSQL = '') THEN '' ELSE ', ' END) || (SELECT JSON_BUILD_OBJECT ('recordID', NULL::bigint,'entities', JSON_BUILD_OBJECT ('sysLoginSession_RefID', varSystemLoginSession::bigint,'sysDataAnnotation', NULL::varchar,'sysDataSetDateTimeTZ', NULL::timestamptz,'sysDataValidityStartDateTimeTZ', NULL::timestamptz,'sysDataValidityFinishDateTimeTZ', NULL::timestamptz,'sysPartitionRemovableRecordKey_RefID', NULL::bigint,'sysBranch_RefID', varInstitutionBranchID::bigint,'sysBaseCurrency_RefID',varBaseCurrencyID::bigint,'name', '254000000000006'::varchar,'iconSource', '97000000000095'::varchar)))::varchar;</v>
+        <v>varSQL := varSQL || (CASE WHEN (varSQL = '') THEN '' ELSE ', ' END) || (SELECT JSON_BUILD_OBJECT ('recordID', NULL::bigint,'entities', JSON_BUILD_OBJECT ('sysLoginSession_RefID', varSystemLoginSession::bigint,'sysDataAnnotation', NULL::varchar,'sysDataSetDateTimeTZ', NULL::timestamptz,'sysDataValidityStartDateTimeTZ', NULL::timestamptz,'sysDataValidityFinishDateTimeTZ', NULL::timestamptz,'sysPartitionRemovableRecordKey_RefID', NULL::bigint,'sysBranch_RefID', varInstitutionBranchID::bigint,'sysBaseCurrency_RefID',varBaseCurrencyID::bigint,'menuGroup_RefID', '254000000000006'::bigint,'menu_RefID', '97000000000095'::bigint)))::varchar;</v>
       </c>
     </row>
     <row r="97" spans="2:11" x14ac:dyDescent="0.2">
@@ -4797,7 +4797,7 @@
       </c>
       <c r="K97" s="2" t="str">
         <f t="shared" si="3"/>
-        <v>varSQL := varSQL || (CASE WHEN (varSQL = '') THEN '' ELSE ', ' END) || (SELECT JSON_BUILD_OBJECT ('recordID', NULL::bigint,'entities', JSON_BUILD_OBJECT ('sysLoginSession_RefID', varSystemLoginSession::bigint,'sysDataAnnotation', NULL::varchar,'sysDataSetDateTimeTZ', NULL::timestamptz,'sysDataValidityStartDateTimeTZ', NULL::timestamptz,'sysDataValidityFinishDateTimeTZ', NULL::timestamptz,'sysPartitionRemovableRecordKey_RefID', NULL::bigint,'sysBranch_RefID', varInstitutionBranchID::bigint,'sysBaseCurrency_RefID',varBaseCurrencyID::bigint,'name', '254000000000006'::varchar,'iconSource', '97000000000096'::varchar)))::varchar;</v>
+        <v>varSQL := varSQL || (CASE WHEN (varSQL = '') THEN '' ELSE ', ' END) || (SELECT JSON_BUILD_OBJECT ('recordID', NULL::bigint,'entities', JSON_BUILD_OBJECT ('sysLoginSession_RefID', varSystemLoginSession::bigint,'sysDataAnnotation', NULL::varchar,'sysDataSetDateTimeTZ', NULL::timestamptz,'sysDataValidityStartDateTimeTZ', NULL::timestamptz,'sysDataValidityFinishDateTimeTZ', NULL::timestamptz,'sysPartitionRemovableRecordKey_RefID', NULL::bigint,'sysBranch_RefID', varInstitutionBranchID::bigint,'sysBaseCurrency_RefID',varBaseCurrencyID::bigint,'menuGroup_RefID', '254000000000006'::bigint,'menu_RefID', '97000000000096'::bigint)))::varchar;</v>
       </c>
     </row>
     <row r="98" spans="2:11" x14ac:dyDescent="0.2">
@@ -4829,7 +4829,7 @@
       </c>
       <c r="K98" s="2" t="str">
         <f t="shared" si="3"/>
-        <v>varSQL := varSQL || (CASE WHEN (varSQL = '') THEN '' ELSE ', ' END) || (SELECT JSON_BUILD_OBJECT ('recordID', NULL::bigint,'entities', JSON_BUILD_OBJECT ('sysLoginSession_RefID', varSystemLoginSession::bigint,'sysDataAnnotation', NULL::varchar,'sysDataSetDateTimeTZ', NULL::timestamptz,'sysDataValidityStartDateTimeTZ', NULL::timestamptz,'sysDataValidityFinishDateTimeTZ', NULL::timestamptz,'sysPartitionRemovableRecordKey_RefID', NULL::bigint,'sysBranch_RefID', varInstitutionBranchID::bigint,'sysBaseCurrency_RefID',varBaseCurrencyID::bigint,'name', '254000000000010'::varchar,'iconSource', '97000000000097'::varchar)))::varchar;</v>
+        <v>varSQL := varSQL || (CASE WHEN (varSQL = '') THEN '' ELSE ', ' END) || (SELECT JSON_BUILD_OBJECT ('recordID', NULL::bigint,'entities', JSON_BUILD_OBJECT ('sysLoginSession_RefID', varSystemLoginSession::bigint,'sysDataAnnotation', NULL::varchar,'sysDataSetDateTimeTZ', NULL::timestamptz,'sysDataValidityStartDateTimeTZ', NULL::timestamptz,'sysDataValidityFinishDateTimeTZ', NULL::timestamptz,'sysPartitionRemovableRecordKey_RefID', NULL::bigint,'sysBranch_RefID', varInstitutionBranchID::bigint,'sysBaseCurrency_RefID',varBaseCurrencyID::bigint,'menuGroup_RefID', '254000000000010'::bigint,'menu_RefID', '97000000000097'::bigint)))::varchar;</v>
       </c>
     </row>
   </sheetData>

</xml_diff>